<commit_message>
Sprint 2: complete radio and coverage validation
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebas\capstone-fwa-rural\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{821015E6-2171-424F-8B99-3B7B1C80A238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378B07AB-9178-4A0B-83A5-93E79A194FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -21,12 +21,25 @@
     <sheet name="Sprint 5" sheetId="6" r:id="rId6"/>
     <sheet name="Sprint 6" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="255">
   <si>
     <t>Product Backlog – Capstone 5G FWA Rural</t>
   </si>
@@ -779,6 +792,18 @@
   </si>
   <si>
     <t>Jhon</t>
+  </si>
+  <si>
+    <t>Bajo</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>Felipe</t>
+  </si>
+  <si>
+    <t>Emanuel</t>
   </si>
 </sst>
 </file>
@@ -1623,15 +1648,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q94"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.69921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.8984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="19.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
@@ -1644,7 +1669,7 @@
     <col min="17" max="17" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="27.9" customHeight="1">
+    <row r="1" spans="1:17" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1667,7 +1692,7 @@
       <c r="P1" s="9"/>
       <c r="Q1" s="9"/>
     </row>
-    <row r="2" spans="1:17" ht="33.9" customHeight="1">
+    <row r="2" spans="1:17" ht="33.950000000000003" customHeight="1">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1711,7 +1736,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="16.8">
+    <row r="4" spans="1:17" ht="16.5">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -1731,28 +1756,28 @@
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(K11:K94,"Finalizado")</f>
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="2">
         <f>COUNTIF(K11:K94,"Pendiente")</f>
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="2">
         <f>SUM(I11:I94)</f>
-        <v>12.5</v>
+        <v>22</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="2">
         <f>SUM(J11:J94)</f>
-        <v>125</v>
+        <v>115.5</v>
       </c>
       <c r="N4" t="s">
         <v>12</v>
@@ -1767,7 +1792,7 @@
       </c>
       <c r="Q4">
         <f>COUNTIFS(D11:D94,2,K11:K94,"Finalizado")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -1787,7 +1812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" ht="15">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1842,7 +1867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="41.4">
+    <row r="10" spans="1:17" ht="45">
       <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
@@ -1883,7 +1908,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" ht="15">
       <c r="A11" s="4" t="s">
         <v>30</v>
       </c>
@@ -1899,8 +1924,12 @@
       <c r="E11" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H11" s="6">
         <v>1</v>
       </c>
@@ -1924,7 +1953,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" ht="15">
       <c r="A12" s="4" t="s">
         <v>33</v>
       </c>
@@ -1940,8 +1969,12 @@
       <c r="E12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
+      <c r="F12" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H12" s="6">
         <v>1</v>
       </c>
@@ -1965,7 +1998,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" ht="29.25">
       <c r="A13" s="4" t="s">
         <v>35</v>
       </c>
@@ -1981,8 +2014,12 @@
       <c r="E13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
+      <c r="F13" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H13" s="6">
         <v>1</v>
       </c>
@@ -2006,7 +2043,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="27.6">
+    <row r="14" spans="1:17" ht="29.25">
       <c r="A14" s="4" t="s">
         <v>37</v>
       </c>
@@ -2022,8 +2059,12 @@
       <c r="E14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
+      <c r="F14" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H14" s="6">
         <v>2</v>
       </c>
@@ -2047,7 +2088,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" ht="15">
       <c r="A15" s="4" t="s">
         <v>39</v>
       </c>
@@ -2063,8 +2104,12 @@
       <c r="E15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
+      <c r="F15" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H15" s="6">
         <v>0.5</v>
       </c>
@@ -2088,7 +2133,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" ht="15">
       <c r="A16" s="4" t="s">
         <v>41</v>
       </c>
@@ -2104,8 +2149,12 @@
       <c r="E16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
+      <c r="F16" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H16" s="6">
         <v>1</v>
       </c>
@@ -2129,7 +2178,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" ht="15">
       <c r="A17" s="4" t="s">
         <v>43</v>
       </c>
@@ -2145,8 +2194,12 @@
       <c r="E17" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
+      <c r="F17" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H17" s="6">
         <v>1</v>
       </c>
@@ -2170,7 +2223,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="27.6">
+    <row r="18" spans="1:13" ht="29.25">
       <c r="A18" s="4" t="s">
         <v>45</v>
       </c>
@@ -2186,8 +2239,12 @@
       <c r="E18" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
+      <c r="F18" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H18" s="6">
         <v>1</v>
       </c>
@@ -2211,7 +2268,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" ht="15">
       <c r="A19" s="4" t="s">
         <v>47</v>
       </c>
@@ -2227,8 +2284,12 @@
       <c r="E19" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
+      <c r="F19" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H19" s="6">
         <v>0.5</v>
       </c>
@@ -2252,7 +2313,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" ht="15">
       <c r="A20" s="4" t="s">
         <v>49</v>
       </c>
@@ -2268,8 +2329,12 @@
       <c r="E20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
+      <c r="F20" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H20" s="6">
         <v>2</v>
       </c>
@@ -2293,7 +2358,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="27.6">
+    <row r="21" spans="1:13" ht="29.25">
       <c r="A21" s="4" t="s">
         <v>51</v>
       </c>
@@ -2309,8 +2374,12 @@
       <c r="E21" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
+      <c r="F21" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H21" s="6">
         <v>1</v>
       </c>
@@ -2335,7 +2404,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" ht="15">
       <c r="A22" s="4" t="s">
         <v>53</v>
       </c>
@@ -2351,8 +2420,12 @@
       <c r="E22" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="F22" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H22" s="6">
         <v>0.5</v>
       </c>
@@ -2377,7 +2450,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="27.6">
+    <row r="23" spans="1:13" ht="29.25">
       <c r="A23" s="4" t="s">
         <v>56</v>
       </c>
@@ -2393,33 +2466,37 @@
       <c r="E23" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
+      <c r="F23" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H23" s="6">
         <v>1</v>
       </c>
-      <c r="I23" s="6" t="str">
+      <c r="I23" s="6">
         <f>IF('Sprint 2'!F10="","",'Sprint 2'!F10)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J23" s="6">
         <f>'Sprint 2'!G10</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" s="4" t="str">
         <f>'Sprint 2'!H10</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L23" s="4" t="str">
         <f>IF('Sprint 2'!C10="","",'Sprint 2'!C10)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M23" s="4" t="str">
         <f>IF('Sprint 2'!K10="","",'Sprint 2'!K10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="27.6">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="29.25">
       <c r="A24" s="4" t="s">
         <v>58</v>
       </c>
@@ -2435,33 +2512,37 @@
       <c r="E24" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
+      <c r="F24" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H24" s="6">
         <v>2</v>
       </c>
-      <c r="I24" s="6" t="str">
+      <c r="I24" s="6">
         <f>IF('Sprint 2'!F11="","",'Sprint 2'!F11)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J24" s="6">
         <f>'Sprint 2'!G11</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K24" s="4" t="str">
         <f>'Sprint 2'!H11</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L24" s="4" t="str">
         <f>IF('Sprint 2'!C11="","",'Sprint 2'!C11)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M24" s="4" t="str">
         <f>IF('Sprint 2'!K11="","",'Sprint 2'!K11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:13" ht="27.6">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="29.25">
       <c r="A25" s="4" t="s">
         <v>60</v>
       </c>
@@ -2482,28 +2563,28 @@
       <c r="H25" s="6">
         <v>2</v>
       </c>
-      <c r="I25" s="6" t="str">
+      <c r="I25" s="6">
         <f>IF('Sprint 2'!F12="","",'Sprint 2'!F12)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J25" s="6">
         <f>'Sprint 2'!G12</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K25" s="4" t="str">
         <f>'Sprint 2'!H12</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L25" s="4" t="str">
         <f>IF('Sprint 2'!C12="","",'Sprint 2'!C12)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M25" s="4" t="str">
         <f>IF('Sprint 2'!K12="","",'Sprint 2'!K12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="15">
       <c r="A26" s="4" t="s">
         <v>62</v>
       </c>
@@ -2524,25 +2605,25 @@
       <c r="H26" s="6">
         <v>1</v>
       </c>
-      <c r="I26" s="6" t="str">
+      <c r="I26" s="6">
         <f>IF('Sprint 2'!F13="","",'Sprint 2'!F13)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J26" s="6">
         <f>'Sprint 2'!G13</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" s="4" t="str">
         <f>'Sprint 2'!H13</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L26" s="4" t="str">
         <f>IF('Sprint 2'!C13="","",'Sprint 2'!C13)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M26" s="4" t="str">
         <f>IF('Sprint 2'!K13="","",'Sprint 2'!K13)</f>
-        <v/>
+        <v>Realizado con éxito</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -2580,7 +2661,7 @@
       </c>
       <c r="L27" s="4" t="str">
         <f>IF('Sprint 2'!C14="","",'Sprint 2'!C14)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M27" s="4" t="str">
         <f>IF('Sprint 2'!K14="","",'Sprint 2'!K14)</f>
@@ -2622,7 +2703,7 @@
       </c>
       <c r="L28" s="4" t="str">
         <f>IF('Sprint 2'!C15="","",'Sprint 2'!C15)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M28" s="4" t="str">
         <f>IF('Sprint 2'!K15="","",'Sprint 2'!K15)</f>
@@ -2664,7 +2745,7 @@
       </c>
       <c r="L29" s="4" t="str">
         <f>IF('Sprint 2'!C16="","",'Sprint 2'!C16)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M29" s="4" t="str">
         <f>IF('Sprint 2'!K16="","",'Sprint 2'!K16)</f>
@@ -2692,28 +2773,28 @@
       <c r="H30" s="6">
         <v>2</v>
       </c>
-      <c r="I30" s="6" t="str">
+      <c r="I30" s="6">
         <f>IF('Sprint 2'!F17="","",'Sprint 2'!F17)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J30" s="6">
         <f>'Sprint 2'!G17</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K30" s="4" t="str">
         <f>'Sprint 2'!H17</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L30" s="4" t="str">
         <f>IF('Sprint 2'!C17="","",'Sprint 2'!C17)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M30" s="4" t="str">
         <f>IF('Sprint 2'!K17="","",'Sprint 2'!K17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:13" ht="27.6">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="28.5">
       <c r="A31" s="4" t="s">
         <v>72</v>
       </c>
@@ -2734,25 +2815,25 @@
       <c r="H31" s="6">
         <v>1.5</v>
       </c>
-      <c r="I31" s="6" t="str">
+      <c r="I31" s="6">
         <f>IF('Sprint 2'!F18="","",'Sprint 2'!F18)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J31" s="6">
         <f>'Sprint 2'!G18</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K31" s="4" t="str">
         <f>'Sprint 2'!H18</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L31" s="4" t="str">
         <f>IF('Sprint 2'!C18="","",'Sprint 2'!C18)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M31" s="4" t="str">
         <f>IF('Sprint 2'!K18="","",'Sprint 2'!K18)</f>
-        <v/>
+        <v>Realizado con éxito</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -2790,14 +2871,14 @@
       </c>
       <c r="L32" s="4" t="str">
         <f>IF('Sprint 2'!C19="","",'Sprint 2'!C19)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M32" s="4" t="str">
         <f>IF('Sprint 2'!K19="","",'Sprint 2'!K19)</f>
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" ht="28.5">
       <c r="A33" s="4" t="s">
         <v>76</v>
       </c>
@@ -2832,14 +2913,14 @@
       </c>
       <c r="L33" s="4" t="str">
         <f>IF('Sprint 2'!C20="","",'Sprint 2'!C20)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M33" s="4" t="str">
         <f>IF('Sprint 2'!K20="","",'Sprint 2'!K20)</f>
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="27.6">
+    <row r="34" spans="1:13" ht="28.5">
       <c r="A34" s="4" t="s">
         <v>78</v>
       </c>
@@ -2874,14 +2955,14 @@
       </c>
       <c r="L34" s="4" t="str">
         <f>IF('Sprint 2'!C21="","",'Sprint 2'!C21)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M34" s="4" t="str">
         <f>IF('Sprint 2'!K21="","",'Sprint 2'!K21)</f>
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" ht="28.5">
       <c r="A35" s="4" t="s">
         <v>80</v>
       </c>
@@ -2916,7 +2997,7 @@
       </c>
       <c r="L35" s="4" t="str">
         <f>IF('Sprint 2'!C22="","",'Sprint 2'!C22)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M35" s="4" t="str">
         <f>IF('Sprint 2'!K22="","",'Sprint 2'!K22)</f>
@@ -2958,7 +3039,7 @@
       </c>
       <c r="L36" s="4" t="str">
         <f>IF('Sprint 2'!C23="","",'Sprint 2'!C23)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M36" s="4" t="str">
         <f>IF('Sprint 2'!K23="","",'Sprint 2'!K23)</f>
@@ -3007,7 +3088,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="27.6">
+    <row r="38" spans="1:13" ht="28.5">
       <c r="A38" s="4" t="s">
         <v>86</v>
       </c>
@@ -3679,7 +3760,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="27.6">
+    <row r="54" spans="1:13" ht="28.5">
       <c r="A54" s="4" t="s">
         <v>118</v>
       </c>
@@ -3721,7 +3802,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="27.6">
+    <row r="55" spans="1:13" ht="28.5">
       <c r="A55" s="4" t="s">
         <v>120</v>
       </c>
@@ -3763,7 +3844,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="27.6">
+    <row r="56" spans="1:13" ht="28.5">
       <c r="A56" s="4" t="s">
         <v>122</v>
       </c>
@@ -3805,7 +3886,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="27.6">
+    <row r="57" spans="1:13" ht="28.5">
       <c r="A57" s="4" t="s">
         <v>124</v>
       </c>
@@ -3889,7 +3970,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="27.6">
+    <row r="59" spans="1:13" ht="28.5">
       <c r="A59" s="4" t="s">
         <v>128</v>
       </c>
@@ -4519,7 +4600,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:13" ht="27.6">
+    <row r="74" spans="1:13" ht="28.5">
       <c r="A74" s="4" t="s">
         <v>158</v>
       </c>
@@ -4813,7 +4894,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:13" ht="27.6">
+    <row r="81" spans="1:13" ht="28.5">
       <c r="A81" s="4" t="s">
         <v>172</v>
       </c>
@@ -4897,7 +4978,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:13" ht="27.6">
+    <row r="83" spans="1:13" ht="28.5">
       <c r="A83" s="4" t="s">
         <v>176</v>
       </c>
@@ -4939,7 +5020,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:13" ht="27.6">
+    <row r="84" spans="1:13" ht="28.5">
       <c r="A84" s="4" t="s">
         <v>178</v>
       </c>
@@ -5149,7 +5230,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="1:13" ht="27.6">
+    <row r="89" spans="1:13" ht="28.5">
       <c r="A89" s="4" t="s">
         <v>188</v>
       </c>
@@ -5191,7 +5272,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="1:13">
+    <row r="90" spans="1:13" ht="28.5">
       <c r="A90" s="4" t="s">
         <v>190</v>
       </c>
@@ -5275,7 +5356,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="1:13" ht="27.6">
+    <row r="92" spans="1:13" ht="28.5">
       <c r="A92" s="4" t="s">
         <v>194</v>
       </c>
@@ -5442,10 +5523,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="22.8984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="51.09765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
@@ -5456,7 +5537,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>200</v>
       </c>
@@ -5471,7 +5552,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -5489,7 +5570,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -5507,7 +5588,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -5525,7 +5606,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -5543,7 +5624,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -5600,7 +5681,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" ht="15">
       <c r="A10" s="4" t="s">
         <v>30</v>
       </c>
@@ -5636,7 +5717,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" ht="15">
       <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
@@ -5672,7 +5753,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" ht="15">
       <c r="A12" s="4" t="s">
         <v>35</v>
       </c>
@@ -5708,7 +5789,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" ht="29.25">
       <c r="A13" s="4" t="s">
         <v>37</v>
       </c>
@@ -5744,7 +5825,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" ht="15">
       <c r="A14" s="4" t="s">
         <v>39</v>
       </c>
@@ -5780,7 +5861,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" ht="15">
       <c r="A15" s="4" t="s">
         <v>41</v>
       </c>
@@ -5816,7 +5897,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" ht="15">
       <c r="A16" s="4" t="s">
         <v>43</v>
       </c>
@@ -5852,7 +5933,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="27.6">
+    <row r="17" spans="1:11" ht="29.25">
       <c r="A17" s="4" t="s">
         <v>45</v>
       </c>
@@ -5888,7 +5969,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" ht="15">
       <c r="A18" s="4" t="s">
         <v>47</v>
       </c>
@@ -5924,7 +6005,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" ht="15">
       <c r="A19" s="4" t="s">
         <v>49</v>
       </c>
@@ -5960,7 +6041,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="27.6">
+    <row r="20" spans="1:11" ht="29.25">
       <c r="A20" s="4" t="s">
         <v>51</v>
       </c>
@@ -5996,7 +6077,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" ht="15">
       <c r="A21" s="4" t="s">
         <v>53</v>
       </c>
@@ -6073,9 +6154,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="25.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -6087,7 +6168,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>222</v>
       </c>
@@ -6102,7 +6183,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -6120,7 +6201,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -6135,10 +6216,10 @@
       </c>
       <c r="H3" s="2">
         <f>COUNTIF(H10:H23,"Finalizado")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="16.8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -6156,7 +6237,7 @@
         <v>23.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -6171,16 +6252,16 @@
       </c>
       <c r="H5" s="2">
         <f>SUM(F10:F23)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="16.8">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
       <c r="H6" s="2">
         <f>SUM(G10:G23)</f>
-        <v>23.5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -6231,118 +6312,160 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="27.6">
+    <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="4" t="s">
         <v>56</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D10" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E10" s="6">
         <v>1</v>
       </c>
-      <c r="F10" s="6"/>
+      <c r="F10" s="6">
+        <v>1</v>
+      </c>
       <c r="G10" s="6">
         <f t="shared" ref="G10:G23" si="0">IF(H10="Finalizado",0,MAX(E10-IF(F10="",0,F10),0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="4"/>
-    </row>
-    <row r="11" spans="1:11" ht="27.6">
+        <v>220</v>
+      </c>
+      <c r="I10" s="5">
+        <v>46263</v>
+      </c>
+      <c r="J10" s="5">
+        <v>46269</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="29.25">
       <c r="A11" s="4" t="s">
         <v>58</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D11" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E11" s="6">
         <v>2</v>
       </c>
-      <c r="F11" s="6"/>
+      <c r="F11" s="6">
+        <v>2</v>
+      </c>
       <c r="G11" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="4"/>
-    </row>
-    <row r="12" spans="1:11" ht="27.6">
+        <v>220</v>
+      </c>
+      <c r="I11" s="5">
+        <v>46263</v>
+      </c>
+      <c r="J11" s="5">
+        <v>46269</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="29.25">
       <c r="A12" s="4" t="s">
         <v>60</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D12" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E12" s="6">
         <v>2</v>
       </c>
-      <c r="F12" s="6"/>
+      <c r="F12" s="6">
+        <v>2</v>
+      </c>
       <c r="G12" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="4"/>
-    </row>
-    <row r="13" spans="1:11">
+        <v>220</v>
+      </c>
+      <c r="I12" s="5">
+        <v>46263</v>
+      </c>
+      <c r="J12" s="5">
+        <v>46269</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15">
       <c r="A13" s="4" t="s">
         <v>62</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D13" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E13" s="6">
         <v>1</v>
       </c>
-      <c r="F13" s="6"/>
+      <c r="F13" s="6">
+        <v>1</v>
+      </c>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="4"/>
-    </row>
-    <row r="14" spans="1:11">
+        <v>220</v>
+      </c>
+      <c r="I13" s="5">
+        <v>46263</v>
+      </c>
+      <c r="J13" s="5">
+        <v>46269</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15">
       <c r="A14" s="4" t="s">
         <v>64</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D14" s="4" t="s">
         <v>32</v>
       </c>
@@ -6368,7 +6491,9 @@
       <c r="B15" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D15" s="4" t="s">
         <v>32</v>
       </c>
@@ -6394,7 +6519,9 @@
       <c r="B16" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D16" s="4" t="s">
         <v>32</v>
       </c>
@@ -6413,57 +6540,77 @@
       <c r="J16" s="5"/>
       <c r="K16" s="4"/>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" ht="15">
       <c r="A17" s="4" t="s">
         <v>70</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D17" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E17" s="6">
         <v>2</v>
       </c>
-      <c r="F17" s="6"/>
+      <c r="F17" s="6">
+        <v>2</v>
+      </c>
       <c r="G17" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="4"/>
-    </row>
-    <row r="18" spans="1:11" ht="27.6">
+        <v>220</v>
+      </c>
+      <c r="I17" s="5">
+        <v>46269</v>
+      </c>
+      <c r="J17" s="5">
+        <v>46270</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="29.25">
       <c r="A18" s="4" t="s">
         <v>72</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D18" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E18" s="6">
         <v>1.5</v>
       </c>
-      <c r="F18" s="6"/>
+      <c r="F18" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G18" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="4"/>
+        <v>220</v>
+      </c>
+      <c r="I18" s="5">
+        <v>46269</v>
+      </c>
+      <c r="J18" s="5">
+        <v>46270</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="4" t="s">
@@ -6472,7 +6619,9 @@
       <c r="B19" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D19" s="4" t="s">
         <v>32</v>
       </c>
@@ -6491,14 +6640,16 @@
       <c r="J19" s="5"/>
       <c r="K19" s="4"/>
     </row>
-    <row r="20" spans="1:11" ht="27.6">
+    <row r="20" spans="1:11" ht="28.5">
       <c r="A20" s="4" t="s">
         <v>76</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D20" s="4" t="s">
         <v>32</v>
       </c>
@@ -6517,14 +6668,16 @@
       <c r="J20" s="5"/>
       <c r="K20" s="4"/>
     </row>
-    <row r="21" spans="1:11" ht="27.6">
+    <row r="21" spans="1:11" ht="28.5">
       <c r="A21" s="4" t="s">
         <v>78</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D21" s="4" t="s">
         <v>55</v>
       </c>
@@ -6543,14 +6696,16 @@
       <c r="J21" s="5"/>
       <c r="K21" s="4"/>
     </row>
-    <row r="22" spans="1:11" ht="27.6">
+    <row r="22" spans="1:11" ht="28.5">
       <c r="A22" s="4" t="s">
         <v>80</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D22" s="4" t="s">
         <v>55</v>
       </c>
@@ -6576,7 +6731,9 @@
       <c r="B23" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D23" s="4" t="s">
         <v>32</v>
       </c>
@@ -6604,9 +6761,9 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:F23">
+  <conditionalFormatting sqref="F14:F16 F19:F23">
     <cfRule type="expression" dxfId="24" priority="5">
-      <formula>AND($H10="Finalizado",$F10="")</formula>
+      <formula>AND($H14="Finalizado",$F14="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:H23">
@@ -6641,9 +6798,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="25.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -6655,7 +6812,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>227</v>
       </c>
@@ -6670,7 +6827,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -6688,7 +6845,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -6706,7 +6863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -6724,7 +6881,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -6742,7 +6899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -6825,7 +6982,7 @@
       <c r="J10" s="5"/>
       <c r="K10" s="4"/>
     </row>
-    <row r="11" spans="1:11" ht="27.6">
+    <row r="11" spans="1:11" ht="28.5">
       <c r="A11" s="4" t="s">
         <v>86</v>
       </c>
@@ -6955,7 +7112,7 @@
       <c r="J15" s="5"/>
       <c r="K15" s="4"/>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" ht="28.5">
       <c r="A16" s="4" t="s">
         <v>96</v>
       </c>
@@ -7033,7 +7190,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="4"/>
     </row>
-    <row r="19" spans="1:11" ht="27.6">
+    <row r="19" spans="1:11" ht="28.5">
       <c r="A19" s="4" t="s">
         <v>102</v>
       </c>
@@ -7105,7 +7262,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7119,7 +7276,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>232</v>
       </c>
@@ -7134,7 +7291,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -7152,7 +7309,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -7170,7 +7327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -7188,7 +7345,7 @@
         <v>22.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -7206,7 +7363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -7445,7 +7602,7 @@
       <c r="J16" s="5"/>
       <c r="K16" s="4"/>
     </row>
-    <row r="17" spans="1:11" ht="27.6">
+    <row r="17" spans="1:11" ht="28.5">
       <c r="A17" s="4" t="s">
         <v>118</v>
       </c>
@@ -7471,7 +7628,7 @@
       <c r="J17" s="5"/>
       <c r="K17" s="4"/>
     </row>
-    <row r="18" spans="1:11" ht="27.6">
+    <row r="18" spans="1:11" ht="28.5">
       <c r="A18" s="4" t="s">
         <v>120</v>
       </c>
@@ -7497,7 +7654,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="4"/>
     </row>
-    <row r="19" spans="1:11" ht="27.6">
+    <row r="19" spans="1:11" ht="28.5">
       <c r="A19" s="4" t="s">
         <v>122</v>
       </c>
@@ -7569,9 +7726,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="23.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -7583,7 +7740,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>236</v>
       </c>
@@ -7598,7 +7755,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -7616,7 +7773,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -7634,7 +7791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -7652,7 +7809,7 @@
         <v>24.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -7670,7 +7827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -7727,7 +7884,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="27.6">
+    <row r="10" spans="1:11" ht="28.5">
       <c r="A10" s="4" t="s">
         <v>124</v>
       </c>
@@ -7779,7 +7936,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11" ht="27.6">
+    <row r="12" spans="1:11" ht="28.5">
       <c r="A12" s="4" t="s">
         <v>128</v>
       </c>
@@ -7831,7 +7988,7 @@
       <c r="J13" s="5"/>
       <c r="K13" s="4"/>
     </row>
-    <row r="14" spans="1:11" ht="27.6">
+    <row r="14" spans="1:11" ht="28.5">
       <c r="A14" s="4" t="s">
         <v>132</v>
       </c>
@@ -8143,7 +8300,7 @@
       <c r="J25" s="5"/>
       <c r="K25" s="4"/>
     </row>
-    <row r="26" spans="1:11" ht="27.6">
+    <row r="26" spans="1:11" ht="28.5">
       <c r="A26" s="4" t="s">
         <v>156</v>
       </c>
@@ -8169,7 +8326,7 @@
       <c r="J26" s="5"/>
       <c r="K26" s="4"/>
     </row>
-    <row r="27" spans="1:11" ht="27.6">
+    <row r="27" spans="1:11" ht="28.5">
       <c r="A27" s="4" t="s">
         <v>158</v>
       </c>
@@ -8241,9 +8398,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="23.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -8255,7 +8412,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>241</v>
       </c>
@@ -8270,7 +8427,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -8288,7 +8445,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -8306,7 +8463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -8324,7 +8481,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -8342,7 +8499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -8451,7 +8608,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" ht="28.5">
       <c r="A12" s="4" t="s">
         <v>164</v>
       </c>
@@ -8555,7 +8712,7 @@
       <c r="J15" s="5"/>
       <c r="K15" s="4"/>
     </row>
-    <row r="16" spans="1:11" ht="27.6">
+    <row r="16" spans="1:11" ht="28.5">
       <c r="A16" s="4" t="s">
         <v>172</v>
       </c>
@@ -8607,7 +8764,7 @@
       <c r="J17" s="5"/>
       <c r="K17" s="4"/>
     </row>
-    <row r="18" spans="1:11" ht="27.6">
+    <row r="18" spans="1:11" ht="28.5">
       <c r="A18" s="4" t="s">
         <v>176</v>
       </c>
@@ -8633,7 +8790,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="4"/>
     </row>
-    <row r="19" spans="1:11" ht="27.6">
+    <row r="19" spans="1:11" ht="28.5">
       <c r="A19" s="4" t="s">
         <v>178</v>
       </c>
@@ -8763,7 +8920,7 @@
       <c r="J23" s="5"/>
       <c r="K23" s="4"/>
     </row>
-    <row r="24" spans="1:11" ht="27.6">
+    <row r="24" spans="1:11" ht="28.5">
       <c r="A24" s="4" t="s">
         <v>188</v>
       </c>
@@ -8789,7 +8946,7 @@
       <c r="J24" s="5"/>
       <c r="K24" s="4"/>
     </row>
-    <row r="25" spans="1:11" ht="27.6">
+    <row r="25" spans="1:11" ht="28.5">
       <c r="A25" s="4" t="s">
         <v>190</v>
       </c>
@@ -8841,7 +8998,7 @@
       <c r="J26" s="5"/>
       <c r="K26" s="4"/>
     </row>
-    <row r="27" spans="1:11" ht="27.6">
+    <row r="27" spans="1:11" ht="28.5">
       <c r="A27" s="4" t="s">
         <v>194</v>
       </c>

</xml_diff>

<commit_message>
Completadas tareas PB17, PB18, PB19 y PB23: Cálculo de capacidad, demanda y sanity checks
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\capstone-fwa-rural\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378B07AB-9178-4A0B-83A5-93E79A194FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80C1A00-4992-4A9C-BF9B-95AF753570CE}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -26,12 +26,6 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -917,11 +911,11 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1670,42 +1664,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.95" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
     </row>
     <row r="2" spans="1:17" ht="33.950000000000003" customHeight="1">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
       <c r="N2" s="3" t="s">
         <v>2</v>
       </c>
@@ -1756,28 +1750,28 @@
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(K11:K94,"Finalizado")</f>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="2">
         <f>COUNTIF(K11:K94,"Pendiente")</f>
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="2">
         <f>SUM(I11:I94)</f>
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="2">
         <f>SUM(J11:J94)</f>
-        <v>115.5</v>
+        <v>108.5</v>
       </c>
       <c r="N4" t="s">
         <v>12</v>
@@ -1792,7 +1786,7 @@
       </c>
       <c r="Q4">
         <f>COUNTIFS(D11:D94,2,K11:K94,"Finalizado")</f>
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -2647,17 +2641,17 @@
       <c r="H27" s="6">
         <v>1.5</v>
       </c>
-      <c r="I27" s="6" t="str">
+      <c r="I27" s="6">
         <f>IF('Sprint 2'!F14="","",'Sprint 2'!F14)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J27" s="6">
         <f>'Sprint 2'!G14</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K27" s="4" t="str">
         <f>'Sprint 2'!H14</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L27" s="4" t="str">
         <f>IF('Sprint 2'!C14="","",'Sprint 2'!C14)</f>
@@ -2689,17 +2683,17 @@
       <c r="H28" s="6">
         <v>2</v>
       </c>
-      <c r="I28" s="6" t="str">
+      <c r="I28" s="6">
         <f>IF('Sprint 2'!F15="","",'Sprint 2'!F15)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J28" s="6">
         <f>'Sprint 2'!G15</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K28" s="4" t="str">
         <f>'Sprint 2'!H15</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L28" s="4" t="str">
         <f>IF('Sprint 2'!C15="","",'Sprint 2'!C15)</f>
@@ -2731,17 +2725,17 @@
       <c r="H29" s="6">
         <v>1.5</v>
       </c>
-      <c r="I29" s="6" t="str">
+      <c r="I29" s="6">
         <f>IF('Sprint 2'!F16="","",'Sprint 2'!F16)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J29" s="6">
         <f>'Sprint 2'!G16</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K29" s="4" t="str">
         <f>'Sprint 2'!H16</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L29" s="4" t="str">
         <f>IF('Sprint 2'!C16="","",'Sprint 2'!C16)</f>
@@ -2752,7 +2746,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" ht="15">
       <c r="A30" s="4" t="s">
         <v>70</v>
       </c>
@@ -2794,7 +2788,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="28.5">
+    <row r="31" spans="1:13" ht="29.25">
       <c r="A31" s="4" t="s">
         <v>72</v>
       </c>
@@ -2899,17 +2893,17 @@
       <c r="H33" s="6">
         <v>2</v>
       </c>
-      <c r="I33" s="6" t="str">
+      <c r="I33" s="6">
         <f>IF('Sprint 2'!F20="","",'Sprint 2'!F20)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J33" s="6">
         <f>'Sprint 2'!G20</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K33" s="4" t="str">
         <f>'Sprint 2'!H20</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L33" s="4" t="str">
         <f>IF('Sprint 2'!C20="","",'Sprint 2'!C20)</f>
@@ -5538,19 +5532,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -5634,17 +5628,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -6169,19 +6163,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -6216,7 +6210,7 @@
       </c>
       <c r="H3" s="2">
         <f>COUNTIF(H10:H23,"Finalizado")</f>
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="16.5">
@@ -6252,7 +6246,7 @@
       </c>
       <c r="H5" s="2">
         <f>SUM(F10:F23)</f>
-        <v>9.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="16.5">
@@ -6261,21 +6255,21 @@
       </c>
       <c r="H6" s="2">
         <f>SUM(G10:G23)</f>
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -6420,7 +6414,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15">
+    <row r="13" spans="1:11" ht="33.75" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>62</v>
       </c>
@@ -6456,7 +6450,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15">
+    <row r="14" spans="1:11" ht="26.25" customHeight="1">
       <c r="A14" s="4" t="s">
         <v>64</v>
       </c>
@@ -6472,19 +6466,25 @@
       <c r="E14" s="6">
         <v>1.5</v>
       </c>
-      <c r="F14" s="6"/>
+      <c r="F14" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I14" s="5">
+        <v>46271</v>
+      </c>
+      <c r="J14" s="5">
+        <v>46273</v>
+      </c>
       <c r="K14" s="4"/>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" ht="15">
       <c r="A15" s="4" t="s">
         <v>66</v>
       </c>
@@ -6500,19 +6500,25 @@
       <c r="E15" s="6">
         <v>2</v>
       </c>
-      <c r="F15" s="6"/>
+      <c r="F15" s="6">
+        <v>2</v>
+      </c>
       <c r="G15" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I15" s="5">
+        <v>46271</v>
+      </c>
+      <c r="J15" s="5">
+        <v>46273</v>
+      </c>
       <c r="K15" s="4"/>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" ht="15">
       <c r="A16" s="4" t="s">
         <v>68</v>
       </c>
@@ -6528,16 +6534,22 @@
       <c r="E16" s="6">
         <v>1.5</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G16" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I16" s="5">
+        <v>46271</v>
+      </c>
+      <c r="J16" s="5">
+        <v>46273</v>
+      </c>
       <c r="K16" s="4"/>
     </row>
     <row r="17" spans="1:11" ht="15">
@@ -6640,7 +6652,7 @@
       <c r="J19" s="5"/>
       <c r="K19" s="4"/>
     </row>
-    <row r="20" spans="1:11" ht="28.5">
+    <row r="20" spans="1:11" ht="29.25">
       <c r="A20" s="4" t="s">
         <v>76</v>
       </c>
@@ -6656,16 +6668,22 @@
       <c r="E20" s="6">
         <v>2</v>
       </c>
-      <c r="F20" s="6"/>
+      <c r="F20" s="6">
+        <v>2</v>
+      </c>
       <c r="G20" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I20" s="5">
+        <v>46271</v>
+      </c>
+      <c r="J20" s="5">
+        <v>46273</v>
+      </c>
       <c r="K20" s="4"/>
     </row>
     <row r="21" spans="1:11" ht="28.5">
@@ -6761,9 +6779,9 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F14:F16 F19:F23">
+  <conditionalFormatting sqref="F19 F21:F23">
     <cfRule type="expression" dxfId="24" priority="5">
-      <formula>AND($H14="Finalizado",$F14="")</formula>
+      <formula>AND($H19="Finalizado",$F19="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:H23">
@@ -6813,19 +6831,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -6909,17 +6927,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -7277,19 +7295,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -7373,17 +7391,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -7741,19 +7759,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -7837,17 +7855,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -8413,19 +8431,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>241</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -8509,17 +8527,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">

</xml_diff>

<commit_message>
docs(sprint2): inicio de tareas PB22, PB24, PB25 y PB26 (Emanuel)
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\capstone-fwa-rural\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Barrios\Desktop\Capstone-Gestion-II\capstone-fwa-rural\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80C1A00-4992-4A9C-BF9B-95AF753570CE}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A49549DE-3850-499A-995A-D47040444985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -33,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="255">
   <si>
     <t>Product Backlog – Capstone 5G FWA Rural</t>
   </si>
@@ -911,11 +917,11 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1642,7 +1648,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q94"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="49.875" bestFit="1" customWidth="1"/>
@@ -1664,42 +1670,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
     </row>
     <row r="2" spans="1:17" ht="33.950000000000003" customHeight="1">
-      <c r="A2" s="9"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
       <c r="N2" s="3" t="s">
         <v>2</v>
       </c>
@@ -2620,7 +2626,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" ht="15">
       <c r="A27" s="4" t="s">
         <v>64</v>
       </c>
@@ -2659,10 +2665,10 @@
       </c>
       <c r="M27" s="4" t="str">
         <f>IF('Sprint 2'!K14="","",'Sprint 2'!K14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="15">
       <c r="A28" s="4" t="s">
         <v>66</v>
       </c>
@@ -2701,10 +2707,10 @@
       </c>
       <c r="M28" s="4" t="str">
         <f>IF('Sprint 2'!K15="","",'Sprint 2'!K15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="15">
       <c r="A29" s="4" t="s">
         <v>68</v>
       </c>
@@ -2743,7 +2749,7 @@
       </c>
       <c r="M29" s="4" t="str">
         <f>IF('Sprint 2'!K16="","",'Sprint 2'!K16)</f>
-        <v/>
+        <v>Realizado con éxito</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="15">
@@ -2872,7 +2878,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="28.5">
+    <row r="33" spans="1:13" ht="29.25">
       <c r="A33" s="4" t="s">
         <v>76</v>
       </c>
@@ -2911,7 +2917,7 @@
       </c>
       <c r="M33" s="4" t="str">
         <f>IF('Sprint 2'!K20="","",'Sprint 2'!K20)</f>
-        <v/>
+        <v>Realizado con éxito</v>
       </c>
     </row>
     <row r="34" spans="1:13" ht="28.5">
@@ -5517,7 +5523,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51.125" bestFit="1" customWidth="1"/>
@@ -5532,19 +5538,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -5628,17 +5634,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -6148,7 +6154,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="25.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -6163,19 +6169,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -6259,17 +6265,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -6482,7 +6488,9 @@
       <c r="J14" s="5">
         <v>46273</v>
       </c>
-      <c r="K14" s="4"/>
+      <c r="K14" s="4" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="15" spans="1:11" ht="15">
       <c r="A15" s="4" t="s">
@@ -6516,7 +6524,9 @@
       <c r="J15" s="5">
         <v>46273</v>
       </c>
-      <c r="K15" s="4"/>
+      <c r="K15" s="4" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="16" spans="1:11" ht="15">
       <c r="A16" s="4" t="s">
@@ -6550,7 +6560,9 @@
       <c r="J16" s="5">
         <v>46273</v>
       </c>
-      <c r="K16" s="4"/>
+      <c r="K16" s="4" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="15">
       <c r="A17" s="4" t="s">
@@ -6648,7 +6660,9 @@
       <c r="H19" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="I19" s="5"/>
+      <c r="I19" s="5">
+        <v>46272</v>
+      </c>
       <c r="J19" s="5"/>
       <c r="K19" s="4"/>
     </row>
@@ -6684,7 +6698,9 @@
       <c r="J20" s="5">
         <v>46273</v>
       </c>
-      <c r="K20" s="4"/>
+      <c r="K20" s="4" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="21" spans="1:11" ht="28.5">
       <c r="A21" s="4" t="s">
@@ -6710,7 +6726,9 @@
       <c r="H21" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="I21" s="5"/>
+      <c r="I21" s="5">
+        <v>46272</v>
+      </c>
       <c r="J21" s="5"/>
       <c r="K21" s="4"/>
     </row>
@@ -6738,7 +6756,9 @@
       <c r="H22" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="I22" s="5"/>
+      <c r="I22" s="5">
+        <v>46272</v>
+      </c>
       <c r="J22" s="5"/>
       <c r="K22" s="4"/>
     </row>
@@ -6766,7 +6786,9 @@
       <c r="H23" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="I23" s="5"/>
+      <c r="I23" s="5">
+        <v>46272</v>
+      </c>
       <c r="J23" s="5"/>
       <c r="K23" s="4"/>
     </row>
@@ -6816,7 +6838,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="25.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -6831,19 +6853,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -6927,17 +6949,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -7280,7 +7302,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7295,19 +7317,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -7391,17 +7413,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -7744,7 +7766,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7759,19 +7781,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -7855,17 +7877,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">
@@ -8416,7 +8438,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -8431,19 +8453,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
     </row>
     <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
@@ -8527,17 +8549,17 @@
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="38.1" customHeight="1">
       <c r="A9" s="3" t="s">

</xml_diff>

<commit_message>
Sprint 2: finalize validated technical model
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Barrios\Desktop\Capstone-Gestion-II\capstone-fwa-rural\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A49549DE-3850-499A-995A-D47040444985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A6990F5-0902-422B-8855-1E31058C11BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="255">
   <si>
     <t>Product Backlog – Capstone 5G FWA Rural</t>
   </si>
@@ -1648,7 +1648,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q94"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="49.875" bestFit="1" customWidth="1"/>
@@ -1756,28 +1756,28 @@
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(K11:K94,"Finalizado")</f>
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="2">
         <f>COUNTIF(K11:K94,"Pendiente")</f>
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="2">
         <f>SUM(I11:I94)</f>
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="2">
         <f>SUM(J11:J94)</f>
-        <v>108.5</v>
+        <v>101.5</v>
       </c>
       <c r="N4" t="s">
         <v>12</v>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="Q4">
         <f>COUNTIFS(D11:D94,2,K11:K94,"Finalizado")</f>
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -2558,8 +2558,12 @@
       <c r="E25" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
+      <c r="F25" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H25" s="6">
         <v>2</v>
       </c>
@@ -2600,8 +2604,12 @@
       <c r="E26" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
+      <c r="F26" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H26" s="6">
         <v>1</v>
       </c>
@@ -2642,8 +2650,12 @@
       <c r="E27" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
+      <c r="F27" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H27" s="6">
         <v>1.5</v>
       </c>
@@ -2684,8 +2696,12 @@
       <c r="E28" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
+      <c r="F28" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H28" s="6">
         <v>2</v>
       </c>
@@ -2726,8 +2742,12 @@
       <c r="E29" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
+      <c r="F29" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H29" s="6">
         <v>1.5</v>
       </c>
@@ -2768,8 +2788,12 @@
       <c r="E30" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
+      <c r="F30" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H30" s="6">
         <v>2</v>
       </c>
@@ -2810,8 +2834,12 @@
       <c r="E31" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
+      <c r="F31" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H31" s="6">
         <v>1.5</v>
       </c>
@@ -2836,7 +2864,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" ht="15">
       <c r="A32" s="4" t="s">
         <v>74</v>
       </c>
@@ -2852,22 +2880,26 @@
       <c r="E32" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
+      <c r="F32" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H32" s="6">
         <v>2</v>
       </c>
-      <c r="I32" s="6" t="str">
+      <c r="I32" s="6">
         <f>IF('Sprint 2'!F19="","",'Sprint 2'!F19)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J32" s="6">
         <f>'Sprint 2'!G19</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K32" s="4" t="str">
         <f>'Sprint 2'!H19</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L32" s="4" t="str">
         <f>IF('Sprint 2'!C19="","",'Sprint 2'!C19)</f>
@@ -2875,7 +2907,7 @@
       </c>
       <c r="M32" s="4" t="str">
         <f>IF('Sprint 2'!K19="","",'Sprint 2'!K19)</f>
-        <v/>
+        <v>Realizado con éxito</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="29.25">
@@ -2894,8 +2926,12 @@
       <c r="E33" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
+      <c r="F33" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H33" s="6">
         <v>2</v>
       </c>
@@ -2920,7 +2956,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="28.5">
+    <row r="34" spans="1:13" ht="29.25">
       <c r="A34" s="4" t="s">
         <v>78</v>
       </c>
@@ -2936,22 +2972,26 @@
       <c r="E34" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
+      <c r="F34" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H34" s="6">
         <v>1.5</v>
       </c>
-      <c r="I34" s="6" t="str">
+      <c r="I34" s="6">
         <f>IF('Sprint 2'!F21="","",'Sprint 2'!F21)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J34" s="6">
         <f>'Sprint 2'!G21</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K34" s="4" t="str">
         <f>'Sprint 2'!H21</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L34" s="4" t="str">
         <f>IF('Sprint 2'!C21="","",'Sprint 2'!C21)</f>
@@ -2959,10 +2999,10 @@
       </c>
       <c r="M34" s="4" t="str">
         <f>IF('Sprint 2'!K21="","",'Sprint 2'!K21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="1:13" ht="28.5">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" ht="29.25">
       <c r="A35" s="4" t="s">
         <v>80</v>
       </c>
@@ -2978,22 +3018,26 @@
       <c r="E35" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
+      <c r="F35" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H35" s="6">
         <v>2</v>
       </c>
-      <c r="I35" s="6" t="str">
+      <c r="I35" s="6">
         <f>IF('Sprint 2'!F22="","",'Sprint 2'!F22)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J35" s="6">
         <f>'Sprint 2'!G22</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K35" s="4" t="str">
         <f>'Sprint 2'!H22</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L35" s="4" t="str">
         <f>IF('Sprint 2'!C22="","",'Sprint 2'!C22)</f>
@@ -3001,10 +3045,10 @@
       </c>
       <c r="M35" s="4" t="str">
         <f>IF('Sprint 2'!K22="","",'Sprint 2'!K22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" ht="15">
       <c r="A36" s="4" t="s">
         <v>82</v>
       </c>
@@ -3020,22 +3064,26 @@
       <c r="E36" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
+      <c r="F36" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H36" s="6">
         <v>1.5</v>
       </c>
-      <c r="I36" s="6" t="str">
+      <c r="I36" s="6">
         <f>IF('Sprint 2'!F23="","",'Sprint 2'!F23)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J36" s="6">
         <f>'Sprint 2'!G23</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K36" s="4" t="str">
         <f>'Sprint 2'!H23</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L36" s="4" t="str">
         <f>IF('Sprint 2'!C23="","",'Sprint 2'!C23)</f>
@@ -3043,7 +3091,7 @@
       </c>
       <c r="M36" s="4" t="str">
         <f>IF('Sprint 2'!K23="","",'Sprint 2'!K23)</f>
-        <v/>
+        <v>Realizado con éxito</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -5523,7 +5571,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51.125" bestFit="1" customWidth="1"/>
@@ -6154,7 +6202,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="25.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -6216,7 +6264,7 @@
       </c>
       <c r="H3" s="2">
         <f>COUNTIF(H10:H23,"Finalizado")</f>
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="16.5">
@@ -6252,7 +6300,7 @@
       </c>
       <c r="H5" s="2">
         <f>SUM(F10:F23)</f>
-        <v>16.5</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="16.5">
@@ -6261,7 +6309,7 @@
       </c>
       <c r="H6" s="2">
         <f>SUM(G10:G23)</f>
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -6636,7 +6684,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" ht="15">
       <c r="A19" s="4" t="s">
         <v>74</v>
       </c>
@@ -6652,19 +6700,25 @@
       <c r="E19" s="6">
         <v>2</v>
       </c>
-      <c r="F19" s="6"/>
+      <c r="F19" s="6">
+        <v>2</v>
+      </c>
       <c r="G19" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I19" s="5">
         <v>46272</v>
       </c>
-      <c r="J19" s="5"/>
-      <c r="K19" s="4"/>
+      <c r="J19" s="5">
+        <v>46274</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="20" spans="1:11" ht="29.25">
       <c r="A20" s="4" t="s">
@@ -6702,7 +6756,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="28.5">
+    <row r="21" spans="1:11" ht="29.25">
       <c r="A21" s="4" t="s">
         <v>78</v>
       </c>
@@ -6718,21 +6772,27 @@
       <c r="E21" s="6">
         <v>1.5</v>
       </c>
-      <c r="F21" s="6"/>
+      <c r="F21" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G21" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I21" s="5">
         <v>46272</v>
       </c>
-      <c r="J21" s="5"/>
-      <c r="K21" s="4"/>
-    </row>
-    <row r="22" spans="1:11" ht="28.5">
+      <c r="J21" s="5">
+        <v>46274</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="29.25">
       <c r="A22" s="4" t="s">
         <v>80</v>
       </c>
@@ -6748,21 +6808,27 @@
       <c r="E22" s="6">
         <v>2</v>
       </c>
-      <c r="F22" s="6"/>
+      <c r="F22" s="6">
+        <v>2</v>
+      </c>
       <c r="G22" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I22" s="5">
         <v>46272</v>
       </c>
-      <c r="J22" s="5"/>
-      <c r="K22" s="4"/>
-    </row>
-    <row r="23" spans="1:11">
+      <c r="J22" s="5">
+        <v>46274</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15">
       <c r="A23" s="4" t="s">
         <v>82</v>
       </c>
@@ -6778,19 +6844,25 @@
       <c r="E23" s="6">
         <v>1.5</v>
       </c>
-      <c r="F23" s="6"/>
+      <c r="F23" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G23" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I23" s="5">
         <v>46272</v>
       </c>
-      <c r="J23" s="5"/>
-      <c r="K23" s="4"/>
+      <c r="J23" s="5">
+        <v>46274</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>247</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -6838,7 +6910,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="25.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7302,7 +7374,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7766,7 +7838,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -8438,7 +8510,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K29"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>

</xml_diff>

<commit_message>
Sprint 3: implementacion inicial de ILS y division de tareas
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A6990F5-0902-422B-8855-1E31058C11BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC23462-A704-4BF5-BD11-BDD8F6C7FD12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="255">
   <si>
     <t>Product Backlog – Capstone 5G FWA Rural</t>
   </si>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="L37" s="4" t="str">
         <f>IF('Sprint 3'!C10="","",'Sprint 3'!C10)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M37" s="4" t="str">
         <f>IF('Sprint 3'!K10="","",'Sprint 3'!K10)</f>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="L38" s="4" t="str">
         <f>IF('Sprint 3'!C11="","",'Sprint 3'!C11)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M38" s="4" t="str">
         <f>IF('Sprint 3'!K11="","",'Sprint 3'!K11)</f>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="L39" s="4" t="str">
         <f>IF('Sprint 3'!C12="","",'Sprint 3'!C12)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M39" s="4" t="str">
         <f>IF('Sprint 3'!K12="","",'Sprint 3'!K12)</f>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="L40" s="4" t="str">
         <f>IF('Sprint 3'!C13="","",'Sprint 3'!C13)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M40" s="4" t="str">
         <f>IF('Sprint 3'!K13="","",'Sprint 3'!K13)</f>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="L41" s="4" t="str">
         <f>IF('Sprint 3'!C14="","",'Sprint 3'!C14)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M41" s="4" t="str">
         <f>IF('Sprint 3'!K14="","",'Sprint 3'!K14)</f>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="L42" s="4" t="str">
         <f>IF('Sprint 3'!C15="","",'Sprint 3'!C15)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M42" s="4" t="str">
         <f>IF('Sprint 3'!K15="","",'Sprint 3'!K15)</f>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="L43" s="4" t="str">
         <f>IF('Sprint 3'!C16="","",'Sprint 3'!C16)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M43" s="4" t="str">
         <f>IF('Sprint 3'!K16="","",'Sprint 3'!K16)</f>
@@ -3423,7 +3423,7 @@
       </c>
       <c r="L44" s="4" t="str">
         <f>IF('Sprint 3'!C17="","",'Sprint 3'!C17)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M44" s="4" t="str">
         <f>IF('Sprint 3'!K17="","",'Sprint 3'!K17)</f>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="L45" s="4" t="str">
         <f>IF('Sprint 3'!C18="","",'Sprint 3'!C18)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M45" s="4" t="str">
         <f>IF('Sprint 3'!K18="","",'Sprint 3'!K18)</f>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="L46" s="4" t="str">
         <f>IF('Sprint 3'!C19="","",'Sprint 3'!C19)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M46" s="4" t="str">
         <f>IF('Sprint 3'!K19="","",'Sprint 3'!K19)</f>
@@ -7075,7 +7075,9 @@
       <c r="B10" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D10" s="4" t="s">
         <v>32</v>
       </c>
@@ -7101,7 +7103,9 @@
       <c r="B11" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D11" s="4" t="s">
         <v>32</v>
       </c>
@@ -7127,7 +7131,9 @@
       <c r="B12" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D12" s="4" t="s">
         <v>32</v>
       </c>
@@ -7153,7 +7159,9 @@
       <c r="B13" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D13" s="4" t="s">
         <v>32</v>
       </c>
@@ -7179,7 +7187,9 @@
       <c r="B14" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D14" s="4" t="s">
         <v>32</v>
       </c>
@@ -7205,7 +7215,9 @@
       <c r="B15" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D15" s="4" t="s">
         <v>32</v>
       </c>
@@ -7231,7 +7243,9 @@
       <c r="B16" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D16" s="4" t="s">
         <v>32</v>
       </c>
@@ -7257,7 +7271,9 @@
       <c r="B17" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D17" s="4" t="s">
         <v>32</v>
       </c>
@@ -7283,7 +7299,9 @@
       <c r="B18" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D18" s="4" t="s">
         <v>55</v>
       </c>
@@ -7309,7 +7327,9 @@
       <c r="B19" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D19" s="4" t="s">
         <v>55</v>
       </c>

</xml_diff>

<commit_message>
Completadas tareas PB30, PB31 y PB34: Evaluación y análisis del Algoritmo ILS
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebas\capstone-fwa-rural\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC23462-A704-4BF5-BD11-BDD8F6C7FD12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{694B7999-8F15-4F57-91B4-E7FAC9015A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="257">
   <si>
     <t>Product Backlog – Capstone 5G FWA Rural</t>
   </si>
@@ -804,6 +804,12 @@
   </si>
   <si>
     <t>Emanuel</t>
+  </si>
+  <si>
+    <t>Validación</t>
+  </si>
+  <si>
+    <t>En Proceso de Revisión</t>
   </si>
 </sst>
 </file>
@@ -1763,21 +1769,21 @@
       </c>
       <c r="H4" s="2">
         <f>COUNTIF(K11:K94,"Pendiente")</f>
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="2">
         <f>SUM(I11:I94)</f>
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="2">
         <f>SUM(J11:J94)</f>
-        <v>101.5</v>
+        <v>96.5</v>
       </c>
       <c r="N4" t="s">
         <v>12</v>
@@ -3241,17 +3247,17 @@
       <c r="H40" s="6">
         <v>2</v>
       </c>
-      <c r="I40" s="6" t="str">
+      <c r="I40" s="6">
         <f>IF('Sprint 3'!F13="","",'Sprint 3'!F13)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J40" s="6">
         <f>'Sprint 3'!G13</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K40" s="4" t="str">
         <f>'Sprint 3'!H13</f>
-        <v>Pendiente</v>
+        <v>Validación</v>
       </c>
       <c r="L40" s="4" t="str">
         <f>IF('Sprint 3'!C13="","",'Sprint 3'!C13)</f>
@@ -3259,7 +3265,7 @@
       </c>
       <c r="M40" s="4" t="str">
         <f>IF('Sprint 3'!K13="","",'Sprint 3'!K13)</f>
-        <v/>
+        <v>En Proceso de Revisión</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -3283,17 +3289,17 @@
       <c r="H41" s="6">
         <v>2</v>
       </c>
-      <c r="I41" s="6" t="str">
+      <c r="I41" s="6">
         <f>IF('Sprint 3'!F14="","",'Sprint 3'!F14)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J41" s="6">
         <f>'Sprint 3'!G14</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K41" s="4" t="str">
         <f>'Sprint 3'!H14</f>
-        <v>Pendiente</v>
+        <v>Validación</v>
       </c>
       <c r="L41" s="4" t="str">
         <f>IF('Sprint 3'!C14="","",'Sprint 3'!C14)</f>
@@ -3301,7 +3307,7 @@
       </c>
       <c r="M41" s="4" t="str">
         <f>IF('Sprint 3'!K14="","",'Sprint 3'!K14)</f>
-        <v/>
+        <v>En Proceso de Revisión</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -3409,17 +3415,17 @@
       <c r="H44" s="6">
         <v>1</v>
       </c>
-      <c r="I44" s="6" t="str">
+      <c r="I44" s="6">
         <f>IF('Sprint 3'!F17="","",'Sprint 3'!F17)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J44" s="6">
         <f>'Sprint 3'!G17</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" s="4" t="str">
         <f>'Sprint 3'!H17</f>
-        <v>Pendiente</v>
+        <v>Validación</v>
       </c>
       <c r="L44" s="4" t="str">
         <f>IF('Sprint 3'!C17="","",'Sprint 3'!C17)</f>
@@ -3427,7 +3433,7 @@
       </c>
       <c r="M44" s="4" t="str">
         <f>IF('Sprint 3'!K17="","",'Sprint 3'!K17)</f>
-        <v/>
+        <v>En Proceso de Revisión</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -7008,7 +7014,7 @@
       </c>
       <c r="H5" s="2">
         <f>SUM(F10:F19)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="16.5">
@@ -7017,7 +7023,7 @@
       </c>
       <c r="H6" s="2">
         <f>SUM(G10:G19)</f>
-        <v>17.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -7152,7 +7158,7 @@
       <c r="J12" s="5"/>
       <c r="K12" s="4"/>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" ht="15">
       <c r="A13" s="4" t="s">
         <v>90</v>
       </c>
@@ -7168,19 +7174,27 @@
       <c r="E13" s="6">
         <v>2</v>
       </c>
-      <c r="F13" s="6"/>
+      <c r="F13" s="6">
+        <v>2</v>
+      </c>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="4"/>
-    </row>
-    <row r="14" spans="1:11">
+        <v>255</v>
+      </c>
+      <c r="I13" s="5">
+        <v>46280</v>
+      </c>
+      <c r="J13" s="5">
+        <v>46282</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15">
       <c r="A14" s="4" t="s">
         <v>92</v>
       </c>
@@ -7196,17 +7210,25 @@
       <c r="E14" s="6">
         <v>2</v>
       </c>
-      <c r="F14" s="6"/>
+      <c r="F14" s="6">
+        <v>2</v>
+      </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="4"/>
+        <v>255</v>
+      </c>
+      <c r="I14" s="5">
+        <v>46280</v>
+      </c>
+      <c r="J14" s="5">
+        <v>46282</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="4" t="s">
@@ -7264,7 +7286,7 @@
       <c r="J16" s="5"/>
       <c r="K16" s="4"/>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" ht="15">
       <c r="A17" s="4" t="s">
         <v>98</v>
       </c>
@@ -7280,17 +7302,25 @@
       <c r="E17" s="6">
         <v>1</v>
       </c>
-      <c r="F17" s="6"/>
+      <c r="F17" s="6">
+        <v>1</v>
+      </c>
       <c r="G17" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="4"/>
+        <v>255</v>
+      </c>
+      <c r="I17" s="5">
+        <v>46280</v>
+      </c>
+      <c r="J17" s="5">
+        <v>46282</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="4" t="s">
@@ -7357,7 +7387,7 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:F19">
+  <conditionalFormatting sqref="F10:F12 F18:F19 F15:F16">
     <cfRule type="expression" dxfId="19" priority="5">
       <formula>AND($H10="Finalizado",$F10="")</formula>
     </cfRule>

</xml_diff>

<commit_message>
Sprint 3: PB32, PB33 y PB36 (Emanuel) - trade-offs y graficas
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebas\capstone-fwa-rural\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Barrios\Desktop\Capstone-Gestion-II\capstone-fwa-rural\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{694B7999-8F15-4F57-91B4-E7FAC9015A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA850A1-92C2-4AB4-843F-36E2740F5755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1654,7 +1654,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q94"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="49.875" bestFit="1" customWidth="1"/>
@@ -3226,7 +3226,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:13" ht="15">
       <c r="A40" s="4" t="s">
         <v>90</v>
       </c>
@@ -3268,7 +3268,7 @@
         <v>En Proceso de Revisión</v>
       </c>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:13" ht="15">
       <c r="A41" s="4" t="s">
         <v>92</v>
       </c>
@@ -3394,7 +3394,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" ht="15">
       <c r="A44" s="4" t="s">
         <v>98</v>
       </c>
@@ -5577,7 +5577,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51.125" bestFit="1" customWidth="1"/>
@@ -6208,7 +6208,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="25.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -6916,7 +6916,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="25.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7254,7 +7254,9 @@
       <c r="H15" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="I15" s="5"/>
+      <c r="I15" s="5">
+        <v>46281</v>
+      </c>
       <c r="J15" s="5"/>
       <c r="K15" s="4"/>
     </row>
@@ -7282,7 +7284,9 @@
       <c r="H16" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="I16" s="5"/>
+      <c r="I16" s="5">
+        <v>46281</v>
+      </c>
       <c r="J16" s="5"/>
       <c r="K16" s="4"/>
     </row>
@@ -7313,7 +7317,7 @@
         <v>255</v>
       </c>
       <c r="I17" s="5">
-        <v>46280</v>
+        <v>46278</v>
       </c>
       <c r="J17" s="5">
         <v>46282</v>
@@ -7374,7 +7378,9 @@
       <c r="H19" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="I19" s="5"/>
+      <c r="I19" s="5">
+        <v>46281</v>
+      </c>
       <c r="J19" s="5"/>
       <c r="K19" s="4"/>
     </row>
@@ -7387,7 +7393,7 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:F12 F18:F19 F15:F16">
+  <conditionalFormatting sqref="F10:F12 F15:F16 F18:F19">
     <cfRule type="expression" dxfId="19" priority="5">
       <formula>AND($H10="Finalizado",$F10="")</formula>
     </cfRule>
@@ -7424,7 +7430,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7888,7 +7894,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -8560,7 +8566,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>

</xml_diff>

<commit_message>
Sprint 3: optimizacion ILS, analisis comparativo y documentacion
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Barrios\Desktop\Capstone-Gestion-II\capstone-fwa-rural\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA850A1-92C2-4AB4-843F-36E2740F5755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A087C97-1FDE-4F2E-813A-55F55F38F477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="256">
   <si>
     <t>Product Backlog – Capstone 5G FWA Rural</t>
   </si>
@@ -806,10 +806,7 @@
     <t>Emanuel</t>
   </si>
   <si>
-    <t>Validación</t>
-  </si>
-  <si>
-    <t>En Proceso de Revisión</t>
+    <t>Terminado con éxito</t>
   </si>
 </sst>
 </file>
@@ -1654,7 +1651,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q94"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="49.875" bestFit="1" customWidth="1"/>
@@ -1762,28 +1759,28 @@
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(K11:K94,"Finalizado")</f>
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="2">
         <f>COUNTIF(K11:K94,"Pendiente")</f>
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="2">
         <f>SUM(I11:I94)</f>
-        <v>41</v>
+        <v>53.5</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="2">
         <f>SUM(J11:J94)</f>
-        <v>96.5</v>
+        <v>84</v>
       </c>
       <c r="N4" t="s">
         <v>12</v>
@@ -1815,7 +1812,7 @@
       </c>
       <c r="Q5">
         <f>COUNTIFS(D11:D94,3,K11:K94,"Finalizado")</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15">
@@ -3100,7 +3097,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" ht="15">
       <c r="A37" s="4" t="s">
         <v>84</v>
       </c>
@@ -3116,22 +3113,26 @@
       <c r="E37" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
+      <c r="F37" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H37" s="6">
         <v>2</v>
       </c>
-      <c r="I37" s="6" t="str">
+      <c r="I37" s="6">
         <f>IF('Sprint 3'!F10="","",'Sprint 3'!F10)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J37" s="6">
         <f>'Sprint 3'!G10</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K37" s="4" t="str">
         <f>'Sprint 3'!H10</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L37" s="4" t="str">
         <f>IF('Sprint 3'!C10="","",'Sprint 3'!C10)</f>
@@ -3139,10 +3140,10 @@
       </c>
       <c r="M37" s="4" t="str">
         <f>IF('Sprint 3'!K10="","",'Sprint 3'!K10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="1:13" ht="28.5">
+        <v>Terminado con éxito</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="29.25">
       <c r="A38" s="4" t="s">
         <v>86</v>
       </c>
@@ -3158,22 +3159,26 @@
       <c r="E38" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
+      <c r="F38" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H38" s="6">
         <v>1.5</v>
       </c>
-      <c r="I38" s="6" t="str">
+      <c r="I38" s="6">
         <f>IF('Sprint 3'!F11="","",'Sprint 3'!F11)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J38" s="6">
         <f>'Sprint 3'!G11</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K38" s="4" t="str">
         <f>'Sprint 3'!H11</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L38" s="4" t="str">
         <f>IF('Sprint 3'!C11="","",'Sprint 3'!C11)</f>
@@ -3181,10 +3186,10 @@
       </c>
       <c r="M38" s="4" t="str">
         <f>IF('Sprint 3'!K11="","",'Sprint 3'!K11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="1:13">
+        <v>Terminado con éxito</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" ht="15">
       <c r="A39" s="4" t="s">
         <v>88</v>
       </c>
@@ -3200,22 +3205,26 @@
       <c r="E39" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
+      <c r="F39" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H39" s="6">
         <v>3</v>
       </c>
-      <c r="I39" s="6" t="str">
+      <c r="I39" s="6">
         <f>IF('Sprint 3'!F12="","",'Sprint 3'!F12)</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="J39" s="6">
         <f>'Sprint 3'!G12</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K39" s="4" t="str">
         <f>'Sprint 3'!H12</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L39" s="4" t="str">
         <f>IF('Sprint 3'!C12="","",'Sprint 3'!C12)</f>
@@ -3223,7 +3232,7 @@
       </c>
       <c r="M39" s="4" t="str">
         <f>IF('Sprint 3'!K12="","",'Sprint 3'!K12)</f>
-        <v/>
+        <v>Terminado con éxito</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="15">
@@ -3242,8 +3251,12 @@
       <c r="E40" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
+      <c r="F40" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H40" s="6">
         <v>2</v>
       </c>
@@ -3257,7 +3270,7 @@
       </c>
       <c r="K40" s="4" t="str">
         <f>'Sprint 3'!H13</f>
-        <v>Validación</v>
+        <v>Finalizado</v>
       </c>
       <c r="L40" s="4" t="str">
         <f>IF('Sprint 3'!C13="","",'Sprint 3'!C13)</f>
@@ -3265,7 +3278,7 @@
       </c>
       <c r="M40" s="4" t="str">
         <f>IF('Sprint 3'!K13="","",'Sprint 3'!K13)</f>
-        <v>En Proceso de Revisión</v>
+        <v>Terminado con éxito</v>
       </c>
     </row>
     <row r="41" spans="1:13" ht="15">
@@ -3284,8 +3297,12 @@
       <c r="E41" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
+      <c r="F41" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H41" s="6">
         <v>2</v>
       </c>
@@ -3299,7 +3316,7 @@
       </c>
       <c r="K41" s="4" t="str">
         <f>'Sprint 3'!H14</f>
-        <v>Validación</v>
+        <v>Finalizado</v>
       </c>
       <c r="L41" s="4" t="str">
         <f>IF('Sprint 3'!C14="","",'Sprint 3'!C14)</f>
@@ -3307,10 +3324,10 @@
       </c>
       <c r="M41" s="4" t="str">
         <f>IF('Sprint 3'!K14="","",'Sprint 3'!K14)</f>
-        <v>En Proceso de Revisión</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13">
+        <v>Terminado con éxito</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="15">
       <c r="A42" s="4" t="s">
         <v>94</v>
       </c>
@@ -3326,22 +3343,26 @@
       <c r="E42" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
+      <c r="F42" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H42" s="6">
         <v>1.5</v>
       </c>
-      <c r="I42" s="6" t="str">
+      <c r="I42" s="6">
         <f>IF('Sprint 3'!F15="","",'Sprint 3'!F15)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J42" s="6">
         <f>'Sprint 3'!G15</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K42" s="4" t="str">
         <f>'Sprint 3'!H15</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L42" s="4" t="str">
         <f>IF('Sprint 3'!C15="","",'Sprint 3'!C15)</f>
@@ -3349,10 +3370,10 @@
       </c>
       <c r="M42" s="4" t="str">
         <f>IF('Sprint 3'!K15="","",'Sprint 3'!K15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="1:13">
+        <v>Terminado con éxito</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="15">
       <c r="A43" s="4" t="s">
         <v>96</v>
       </c>
@@ -3368,22 +3389,26 @@
       <c r="E43" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
+      <c r="F43" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H43" s="6">
         <v>1.5</v>
       </c>
-      <c r="I43" s="6" t="str">
+      <c r="I43" s="6">
         <f>IF('Sprint 3'!F16="","",'Sprint 3'!F16)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J43" s="6">
         <f>'Sprint 3'!G16</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K43" s="4" t="str">
         <f>'Sprint 3'!H16</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L43" s="4" t="str">
         <f>IF('Sprint 3'!C16="","",'Sprint 3'!C16)</f>
@@ -3391,7 +3416,7 @@
       </c>
       <c r="M43" s="4" t="str">
         <f>IF('Sprint 3'!K16="","",'Sprint 3'!K16)</f>
-        <v/>
+        <v>Terminado con éxito</v>
       </c>
     </row>
     <row r="44" spans="1:13" ht="15">
@@ -3410,8 +3435,12 @@
       <c r="E44" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
+      <c r="F44" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H44" s="6">
         <v>1</v>
       </c>
@@ -3425,7 +3454,7 @@
       </c>
       <c r="K44" s="4" t="str">
         <f>'Sprint 3'!H17</f>
-        <v>Validación</v>
+        <v>Finalizado</v>
       </c>
       <c r="L44" s="4" t="str">
         <f>IF('Sprint 3'!C17="","",'Sprint 3'!C17)</f>
@@ -3433,10 +3462,10 @@
       </c>
       <c r="M44" s="4" t="str">
         <f>IF('Sprint 3'!K17="","",'Sprint 3'!K17)</f>
-        <v>En Proceso de Revisión</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13">
+        <v>Terminado con éxito</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" ht="15">
       <c r="A45" s="4" t="s">
         <v>100</v>
       </c>
@@ -3452,22 +3481,26 @@
       <c r="E45" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
+      <c r="F45" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H45" s="6">
         <v>1.5</v>
       </c>
-      <c r="I45" s="6" t="str">
+      <c r="I45" s="6">
         <f>IF('Sprint 3'!F18="","",'Sprint 3'!F18)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J45" s="6">
         <f>'Sprint 3'!G18</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K45" s="4" t="str">
         <f>'Sprint 3'!H18</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L45" s="4" t="str">
         <f>IF('Sprint 3'!C18="","",'Sprint 3'!C18)</f>
@@ -3475,10 +3508,10 @@
       </c>
       <c r="M45" s="4" t="str">
         <f>IF('Sprint 3'!K18="","",'Sprint 3'!K18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="1:13">
+        <v>Terminado con éxito</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" ht="15">
       <c r="A46" s="4" t="s">
         <v>102</v>
       </c>
@@ -3494,22 +3527,26 @@
       <c r="E46" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
+      <c r="F46" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="H46" s="6">
         <v>1.5</v>
       </c>
-      <c r="I46" s="6" t="str">
+      <c r="I46" s="6">
         <f>IF('Sprint 3'!F19="","",'Sprint 3'!F19)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J46" s="6">
         <f>'Sprint 3'!G19</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K46" s="4" t="str">
         <f>'Sprint 3'!H19</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L46" s="4" t="str">
         <f>IF('Sprint 3'!C19="","",'Sprint 3'!C19)</f>
@@ -3517,7 +3554,7 @@
       </c>
       <c r="M46" s="4" t="str">
         <f>IF('Sprint 3'!K19="","",'Sprint 3'!K19)</f>
-        <v/>
+        <v>Terminado con éxito</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -5577,7 +5614,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51.125" bestFit="1" customWidth="1"/>
@@ -6208,7 +6245,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="25.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -6916,7 +6953,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="25.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -6978,7 +7015,7 @@
       </c>
       <c r="H3" s="2">
         <f>COUNTIF(H10:H19,"Finalizado")</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="16.5">
@@ -7014,7 +7051,7 @@
       </c>
       <c r="H5" s="2">
         <f>SUM(F10:F19)</f>
-        <v>5</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="16.5">
@@ -7023,7 +7060,7 @@
       </c>
       <c r="H6" s="2">
         <f>SUM(G10:G19)</f>
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -7074,7 +7111,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" ht="15">
       <c r="A10" s="4" t="s">
         <v>84</v>
       </c>
@@ -7090,19 +7127,27 @@
       <c r="E10" s="6">
         <v>2</v>
       </c>
-      <c r="F10" s="6"/>
+      <c r="F10" s="6">
+        <v>2</v>
+      </c>
       <c r="G10" s="6">
         <f t="shared" ref="G10:G19" si="0">IF(H10="Finalizado",0,MAX(E10-IF(F10="",0,F10),0))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="4"/>
-    </row>
-    <row r="11" spans="1:11" ht="28.5">
+        <v>220</v>
+      </c>
+      <c r="I10" s="5">
+        <v>46277</v>
+      </c>
+      <c r="J10" s="5">
+        <v>46280</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="29.25">
       <c r="A11" s="4" t="s">
         <v>86</v>
       </c>
@@ -7118,19 +7163,27 @@
       <c r="E11" s="6">
         <v>1.5</v>
       </c>
-      <c r="F11" s="6"/>
+      <c r="F11" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G11" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="4"/>
-    </row>
-    <row r="12" spans="1:11">
+        <v>220</v>
+      </c>
+      <c r="I11" s="5">
+        <v>46277</v>
+      </c>
+      <c r="J11" s="5">
+        <v>46280</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15">
       <c r="A12" s="4" t="s">
         <v>88</v>
       </c>
@@ -7146,17 +7199,25 @@
       <c r="E12" s="6">
         <v>3</v>
       </c>
-      <c r="F12" s="6"/>
+      <c r="F12" s="6">
+        <v>3</v>
+      </c>
       <c r="G12" s="6">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="4"/>
+        <v>220</v>
+      </c>
+      <c r="I12" s="5">
+        <v>46277</v>
+      </c>
+      <c r="J12" s="5">
+        <v>46280</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="13" spans="1:11" ht="15">
       <c r="A13" s="4" t="s">
@@ -7182,7 +7243,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
       <c r="I13" s="5">
         <v>46280</v>
@@ -7191,7 +7252,7 @@
         <v>46282</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="15">
@@ -7218,7 +7279,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
       <c r="I14" s="5">
         <v>46280</v>
@@ -7227,7 +7288,7 @@
         <v>46282</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -7246,19 +7307,25 @@
       <c r="E15" s="6">
         <v>1.5</v>
       </c>
-      <c r="F15" s="6"/>
+      <c r="F15" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G15" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I15" s="5">
         <v>46281</v>
       </c>
-      <c r="J15" s="5"/>
-      <c r="K15" s="4"/>
+      <c r="J15" s="5">
+        <v>46285</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="16" spans="1:11" ht="28.5">
       <c r="A16" s="4" t="s">
@@ -7276,19 +7343,25 @@
       <c r="E16" s="6">
         <v>1.5</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G16" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I16" s="5">
         <v>46281</v>
       </c>
-      <c r="J16" s="5"/>
-      <c r="K16" s="4"/>
+      <c r="J16" s="5">
+        <v>46285</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="15">
       <c r="A17" s="4" t="s">
@@ -7314,16 +7387,16 @@
         <v>0</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>255</v>
+        <v>220</v>
       </c>
       <c r="I17" s="5">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="J17" s="5">
         <v>46282</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -7342,17 +7415,25 @@
       <c r="E18" s="6">
         <v>1.5</v>
       </c>
-      <c r="F18" s="6"/>
+      <c r="F18" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G18" s="6">
-        <f t="shared" si="0"/>
-        <v>1.5</v>
+        <f>IF(H18="Finalizado",0,MAX(E18-IF(F18="",0,F18),0))</f>
+        <v>0</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="4"/>
+        <v>220</v>
+      </c>
+      <c r="I18" s="5">
+        <v>46277</v>
+      </c>
+      <c r="J18" s="5">
+        <v>46285</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="19" spans="1:11" ht="28.5">
       <c r="A19" s="4" t="s">
@@ -7370,19 +7451,25 @@
       <c r="E19" s="6">
         <v>1.5</v>
       </c>
-      <c r="F19" s="6"/>
+      <c r="F19" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G19" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I19" s="5">
         <v>46281</v>
       </c>
-      <c r="J19" s="5"/>
-      <c r="K19" s="4"/>
+      <c r="J19" s="5">
+        <v>46285</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>255</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -7393,11 +7480,6 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:F12 F15:F16 F18:F19">
-    <cfRule type="expression" dxfId="19" priority="5">
-      <formula>AND($H10="Finalizado",$F10="")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H10:H19">
     <cfRule type="expression" dxfId="18" priority="1">
       <formula>$H10="Finalizado"</formula>
@@ -7430,7 +7512,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7894,7 +7976,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -8566,7 +8648,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K29"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>

</xml_diff>

<commit_message>
Asignacion de Tareas para sprint 5
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebas\capstone-fwa-rural\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A087C97-1FDE-4F2E-813A-55F55F38F477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6035BB44-1FC1-4B68-82AE-D0A1C6C600E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="257">
   <si>
     <t>Product Backlog – Capstone 5G FWA Rural</t>
   </si>
@@ -807,6 +807,9 @@
   </si>
   <si>
     <t>Terminado con éxito</t>
+  </si>
+  <si>
+    <t>Validación</t>
   </si>
 </sst>
 </file>
@@ -933,7 +936,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="34">
+  <dxfs count="33">
     <dxf>
       <font>
         <b/>
@@ -1140,17 +1143,6 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1651,15 +1643,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q94"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="14.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.8984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.59765625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.59765625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="19.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
@@ -1672,7 +1664,7 @@
     <col min="17" max="17" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="27.95" customHeight="1">
+    <row r="1" spans="1:17" ht="27.9" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1695,7 +1687,7 @@
       <c r="P1" s="9"/>
       <c r="Q1" s="9"/>
     </row>
-    <row r="2" spans="1:17" ht="33.950000000000003" customHeight="1">
+    <row r="2" spans="1:17" ht="33.9" customHeight="1">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1739,7 +1731,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="16.5">
+    <row r="4" spans="1:17" ht="16.8">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -1766,21 +1758,21 @@
       </c>
       <c r="H4" s="2">
         <f>COUNTIF(K11:K94,"Pendiente")</f>
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="2">
         <f>SUM(I11:I94)</f>
-        <v>53.5</v>
+        <v>63.5</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="2">
         <f>SUM(J11:J94)</f>
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="N4" t="s">
         <v>12</v>
@@ -1815,7 +1807,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15">
+    <row r="6" spans="1:17">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1870,7 +1862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="45">
+    <row r="10" spans="1:17" ht="41.4">
       <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
@@ -1911,7 +1903,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="15">
+    <row r="11" spans="1:17">
       <c r="A11" s="4" t="s">
         <v>30</v>
       </c>
@@ -1956,7 +1948,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="15">
+    <row r="12" spans="1:17">
       <c r="A12" s="4" t="s">
         <v>33</v>
       </c>
@@ -2001,7 +1993,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="29.25">
+    <row r="13" spans="1:17">
       <c r="A13" s="4" t="s">
         <v>35</v>
       </c>
@@ -2046,7 +2038,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="29.25">
+    <row r="14" spans="1:17" ht="27.6">
       <c r="A14" s="4" t="s">
         <v>37</v>
       </c>
@@ -2091,7 +2083,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="15">
+    <row r="15" spans="1:17">
       <c r="A15" s="4" t="s">
         <v>39</v>
       </c>
@@ -2136,7 +2128,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="15">
+    <row r="16" spans="1:17">
       <c r="A16" s="4" t="s">
         <v>41</v>
       </c>
@@ -2181,7 +2173,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="15">
+    <row r="17" spans="1:13">
       <c r="A17" s="4" t="s">
         <v>43</v>
       </c>
@@ -2226,7 +2218,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="29.25">
+    <row r="18" spans="1:13" ht="27.6">
       <c r="A18" s="4" t="s">
         <v>45</v>
       </c>
@@ -2271,7 +2263,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="15">
+    <row r="19" spans="1:13">
       <c r="A19" s="4" t="s">
         <v>47</v>
       </c>
@@ -2316,7 +2308,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="15">
+    <row r="20" spans="1:13">
       <c r="A20" s="4" t="s">
         <v>49</v>
       </c>
@@ -2361,7 +2353,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="29.25">
+    <row r="21" spans="1:13" ht="27.6">
       <c r="A21" s="4" t="s">
         <v>51</v>
       </c>
@@ -2407,7 +2399,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="15">
+    <row r="22" spans="1:13">
       <c r="A22" s="4" t="s">
         <v>53</v>
       </c>
@@ -2453,7 +2445,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="29.25">
+    <row r="23" spans="1:13" ht="27.6">
       <c r="A23" s="4" t="s">
         <v>56</v>
       </c>
@@ -2499,7 +2491,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="29.25">
+    <row r="24" spans="1:13" ht="27.6">
       <c r="A24" s="4" t="s">
         <v>58</v>
       </c>
@@ -2545,7 +2537,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="29.25">
+    <row r="25" spans="1:13" ht="27.6">
       <c r="A25" s="4" t="s">
         <v>60</v>
       </c>
@@ -2591,7 +2583,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="15">
+    <row r="26" spans="1:13">
       <c r="A26" s="4" t="s">
         <v>62</v>
       </c>
@@ -2637,7 +2629,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="15">
+    <row r="27" spans="1:13">
       <c r="A27" s="4" t="s">
         <v>64</v>
       </c>
@@ -2683,7 +2675,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="15">
+    <row r="28" spans="1:13">
       <c r="A28" s="4" t="s">
         <v>66</v>
       </c>
@@ -2729,7 +2721,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="15">
+    <row r="29" spans="1:13">
       <c r="A29" s="4" t="s">
         <v>68</v>
       </c>
@@ -2775,7 +2767,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="15">
+    <row r="30" spans="1:13">
       <c r="A30" s="4" t="s">
         <v>70</v>
       </c>
@@ -2821,7 +2813,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="29.25">
+    <row r="31" spans="1:13" ht="27.6">
       <c r="A31" s="4" t="s">
         <v>72</v>
       </c>
@@ -2867,7 +2859,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="15">
+    <row r="32" spans="1:13">
       <c r="A32" s="4" t="s">
         <v>74</v>
       </c>
@@ -2913,7 +2905,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="29.25">
+    <row r="33" spans="1:13">
       <c r="A33" s="4" t="s">
         <v>76</v>
       </c>
@@ -2959,7 +2951,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="29.25">
+    <row r="34" spans="1:13" ht="27.6">
       <c r="A34" s="4" t="s">
         <v>78</v>
       </c>
@@ -3005,7 +2997,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="29.25">
+    <row r="35" spans="1:13">
       <c r="A35" s="4" t="s">
         <v>80</v>
       </c>
@@ -3051,7 +3043,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="15">
+    <row r="36" spans="1:13">
       <c r="A36" s="4" t="s">
         <v>82</v>
       </c>
@@ -3097,7 +3089,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="15">
+    <row r="37" spans="1:13">
       <c r="A37" s="4" t="s">
         <v>84</v>
       </c>
@@ -3143,7 +3135,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="29.25">
+    <row r="38" spans="1:13" ht="27.6">
       <c r="A38" s="4" t="s">
         <v>86</v>
       </c>
@@ -3189,7 +3181,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="15">
+    <row r="39" spans="1:13">
       <c r="A39" s="4" t="s">
         <v>88</v>
       </c>
@@ -3235,7 +3227,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="15">
+    <row r="40" spans="1:13">
       <c r="A40" s="4" t="s">
         <v>90</v>
       </c>
@@ -3281,7 +3273,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="15">
+    <row r="41" spans="1:13">
       <c r="A41" s="4" t="s">
         <v>92</v>
       </c>
@@ -3327,7 +3319,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="15">
+    <row r="42" spans="1:13">
       <c r="A42" s="4" t="s">
         <v>94</v>
       </c>
@@ -3373,7 +3365,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="15">
+    <row r="43" spans="1:13">
       <c r="A43" s="4" t="s">
         <v>96</v>
       </c>
@@ -3419,7 +3411,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="15">
+    <row r="44" spans="1:13">
       <c r="A44" s="4" t="s">
         <v>98</v>
       </c>
@@ -3465,7 +3457,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="15">
+    <row r="45" spans="1:13">
       <c r="A45" s="4" t="s">
         <v>100</v>
       </c>
@@ -3511,7 +3503,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="15">
+    <row r="46" spans="1:13">
       <c r="A46" s="4" t="s">
         <v>102</v>
       </c>
@@ -3592,7 +3584,7 @@
       </c>
       <c r="L47" s="4" t="str">
         <f>IF('Sprint 4'!C10="","",'Sprint 4'!C10)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M47" s="4" t="str">
         <f>IF('Sprint 4'!K10="","",'Sprint 4'!K10)</f>
@@ -3634,7 +3626,7 @@
       </c>
       <c r="L48" s="4" t="str">
         <f>IF('Sprint 4'!C11="","",'Sprint 4'!C11)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M48" s="4" t="str">
         <f>IF('Sprint 4'!K11="","",'Sprint 4'!K11)</f>
@@ -3662,21 +3654,21 @@
       <c r="H49" s="6">
         <v>2</v>
       </c>
-      <c r="I49" s="6" t="str">
+      <c r="I49" s="6">
         <f>IF('Sprint 4'!F12="","",'Sprint 4'!F12)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J49" s="6">
         <f>'Sprint 4'!G12</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K49" s="4" t="str">
         <f>'Sprint 4'!H12</f>
-        <v>Pendiente</v>
+        <v>Validación</v>
       </c>
       <c r="L49" s="4" t="str">
         <f>IF('Sprint 4'!C12="","",'Sprint 4'!C12)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M49" s="4" t="str">
         <f>IF('Sprint 4'!K12="","",'Sprint 4'!K12)</f>
@@ -3704,21 +3696,21 @@
       <c r="H50" s="6">
         <v>2</v>
       </c>
-      <c r="I50" s="6" t="str">
+      <c r="I50" s="6">
         <f>IF('Sprint 4'!F13="","",'Sprint 4'!F13)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J50" s="6">
         <f>'Sprint 4'!G13</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K50" s="4" t="str">
         <f>'Sprint 4'!H13</f>
-        <v>Pendiente</v>
+        <v>Validación</v>
       </c>
       <c r="L50" s="4" t="str">
         <f>IF('Sprint 4'!C13="","",'Sprint 4'!C13)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M50" s="4" t="str">
         <f>IF('Sprint 4'!K13="","",'Sprint 4'!K13)</f>
@@ -3746,21 +3738,21 @@
       <c r="H51" s="6">
         <v>2</v>
       </c>
-      <c r="I51" s="6" t="str">
+      <c r="I51" s="6">
         <f>IF('Sprint 4'!F14="","",'Sprint 4'!F14)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J51" s="6">
         <f>'Sprint 4'!G14</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K51" s="4" t="str">
         <f>'Sprint 4'!H14</f>
-        <v>Pendiente</v>
+        <v>Validación</v>
       </c>
       <c r="L51" s="4" t="str">
         <f>IF('Sprint 4'!C14="","",'Sprint 4'!C14)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M51" s="4" t="str">
         <f>IF('Sprint 4'!K14="","",'Sprint 4'!K14)</f>
@@ -3788,21 +3780,21 @@
       <c r="H52" s="6">
         <v>2</v>
       </c>
-      <c r="I52" s="6" t="str">
+      <c r="I52" s="6">
         <f>IF('Sprint 4'!F15="","",'Sprint 4'!F15)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J52" s="6">
         <f>'Sprint 4'!G15</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K52" s="4" t="str">
         <f>'Sprint 4'!H15</f>
-        <v>Pendiente</v>
+        <v>Validación</v>
       </c>
       <c r="L52" s="4" t="str">
         <f>IF('Sprint 4'!C15="","",'Sprint 4'!C15)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M52" s="4" t="str">
         <f>IF('Sprint 4'!K15="","",'Sprint 4'!K15)</f>
@@ -3830,28 +3822,28 @@
       <c r="H53" s="6">
         <v>2</v>
       </c>
-      <c r="I53" s="6" t="str">
+      <c r="I53" s="6">
         <f>IF('Sprint 4'!F16="","",'Sprint 4'!F16)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J53" s="6">
         <f>'Sprint 4'!G16</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K53" s="4" t="str">
         <f>'Sprint 4'!H16</f>
-        <v>Pendiente</v>
+        <v>Validación</v>
       </c>
       <c r="L53" s="4" t="str">
         <f>IF('Sprint 4'!C16="","",'Sprint 4'!C16)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M53" s="4" t="str">
         <f>IF('Sprint 4'!K16="","",'Sprint 4'!K16)</f>
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="28.5">
+    <row r="54" spans="1:13" ht="27.6">
       <c r="A54" s="4" t="s">
         <v>118</v>
       </c>
@@ -3893,7 +3885,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="28.5">
+    <row r="55" spans="1:13" ht="27.6">
       <c r="A55" s="4" t="s">
         <v>120</v>
       </c>
@@ -3935,7 +3927,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="28.5">
+    <row r="56" spans="1:13" ht="27.6">
       <c r="A56" s="4" t="s">
         <v>122</v>
       </c>
@@ -3977,7 +3969,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="28.5">
+    <row r="57" spans="1:13" ht="27.6">
       <c r="A57" s="4" t="s">
         <v>124</v>
       </c>
@@ -4012,7 +4004,7 @@
       </c>
       <c r="L57" s="4" t="str">
         <f>IF('Sprint 5'!C10="","",'Sprint 5'!C10)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M57" s="4" t="str">
         <f>IF('Sprint 5'!K10="","",'Sprint 5'!K10)</f>
@@ -4054,14 +4046,14 @@
       </c>
       <c r="L58" s="4" t="str">
         <f>IF('Sprint 5'!C11="","",'Sprint 5'!C11)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M58" s="4" t="str">
         <f>IF('Sprint 5'!K11="","",'Sprint 5'!K11)</f>
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="28.5">
+    <row r="59" spans="1:13" ht="27.6">
       <c r="A59" s="4" t="s">
         <v>128</v>
       </c>
@@ -4096,7 +4088,7 @@
       </c>
       <c r="L59" s="4" t="str">
         <f>IF('Sprint 5'!C12="","",'Sprint 5'!C12)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M59" s="4" t="str">
         <f>IF('Sprint 5'!K12="","",'Sprint 5'!K12)</f>
@@ -4138,7 +4130,7 @@
       </c>
       <c r="L60" s="4" t="str">
         <f>IF('Sprint 5'!C13="","",'Sprint 5'!C13)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M60" s="4" t="str">
         <f>IF('Sprint 5'!K13="","",'Sprint 5'!K13)</f>
@@ -4180,7 +4172,7 @@
       </c>
       <c r="L61" s="4" t="str">
         <f>IF('Sprint 5'!C14="","",'Sprint 5'!C14)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M61" s="4" t="str">
         <f>IF('Sprint 5'!K14="","",'Sprint 5'!K14)</f>
@@ -4222,7 +4214,7 @@
       </c>
       <c r="L62" s="4" t="str">
         <f>IF('Sprint 5'!C15="","",'Sprint 5'!C15)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M62" s="4" t="str">
         <f>IF('Sprint 5'!K15="","",'Sprint 5'!K15)</f>
@@ -4264,7 +4256,7 @@
       </c>
       <c r="L63" s="4" t="str">
         <f>IF('Sprint 5'!C16="","",'Sprint 5'!C16)</f>
-        <v/>
+        <v>Felipe</v>
       </c>
       <c r="M63" s="4" t="str">
         <f>IF('Sprint 5'!K16="","",'Sprint 5'!K16)</f>
@@ -4306,7 +4298,7 @@
       </c>
       <c r="L64" s="4" t="str">
         <f>IF('Sprint 5'!C17="","",'Sprint 5'!C17)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M64" s="4" t="str">
         <f>IF('Sprint 5'!K17="","",'Sprint 5'!K17)</f>
@@ -4348,7 +4340,7 @@
       </c>
       <c r="L65" s="4" t="str">
         <f>IF('Sprint 5'!C18="","",'Sprint 5'!C18)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M65" s="4" t="str">
         <f>IF('Sprint 5'!K18="","",'Sprint 5'!K18)</f>
@@ -4390,7 +4382,7 @@
       </c>
       <c r="L66" s="4" t="str">
         <f>IF('Sprint 5'!C19="","",'Sprint 5'!C19)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M66" s="4" t="str">
         <f>IF('Sprint 5'!K19="","",'Sprint 5'!K19)</f>
@@ -4432,7 +4424,7 @@
       </c>
       <c r="L67" s="4" t="str">
         <f>IF('Sprint 5'!C20="","",'Sprint 5'!C20)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M67" s="4" t="str">
         <f>IF('Sprint 5'!K20="","",'Sprint 5'!K20)</f>
@@ -4474,7 +4466,7 @@
       </c>
       <c r="L68" s="4" t="str">
         <f>IF('Sprint 5'!C21="","",'Sprint 5'!C21)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M68" s="4" t="str">
         <f>IF('Sprint 5'!K21="","",'Sprint 5'!K21)</f>
@@ -4516,7 +4508,7 @@
       </c>
       <c r="L69" s="4" t="str">
         <f>IF('Sprint 5'!C22="","",'Sprint 5'!C22)</f>
-        <v/>
+        <v>Emanuel</v>
       </c>
       <c r="M69" s="4" t="str">
         <f>IF('Sprint 5'!K22="","",'Sprint 5'!K22)</f>
@@ -4558,7 +4550,7 @@
       </c>
       <c r="L70" s="4" t="str">
         <f>IF('Sprint 5'!C23="","",'Sprint 5'!C23)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M70" s="4" t="str">
         <f>IF('Sprint 5'!K23="","",'Sprint 5'!K23)</f>
@@ -4600,7 +4592,7 @@
       </c>
       <c r="L71" s="4" t="str">
         <f>IF('Sprint 5'!C24="","",'Sprint 5'!C24)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M71" s="4" t="str">
         <f>IF('Sprint 5'!K24="","",'Sprint 5'!K24)</f>
@@ -4642,7 +4634,7 @@
       </c>
       <c r="L72" s="4" t="str">
         <f>IF('Sprint 5'!C25="","",'Sprint 5'!C25)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M72" s="4" t="str">
         <f>IF('Sprint 5'!K25="","",'Sprint 5'!K25)</f>
@@ -4684,14 +4676,14 @@
       </c>
       <c r="L73" s="4" t="str">
         <f>IF('Sprint 5'!C26="","",'Sprint 5'!C26)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M73" s="4" t="str">
         <f>IF('Sprint 5'!K26="","",'Sprint 5'!K26)</f>
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:13" ht="28.5">
+    <row r="74" spans="1:13" ht="27.6">
       <c r="A74" s="4" t="s">
         <v>158</v>
       </c>
@@ -4726,7 +4718,7 @@
       </c>
       <c r="L74" s="4" t="str">
         <f>IF('Sprint 5'!C27="","",'Sprint 5'!C27)</f>
-        <v/>
+        <v>Jhon</v>
       </c>
       <c r="M74" s="4" t="str">
         <f>IF('Sprint 5'!K27="","",'Sprint 5'!K27)</f>
@@ -4985,7 +4977,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:13" ht="28.5">
+    <row r="81" spans="1:13" ht="27.6">
       <c r="A81" s="4" t="s">
         <v>172</v>
       </c>
@@ -5069,7 +5061,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:13" ht="28.5">
+    <row r="83" spans="1:13" ht="27.6">
       <c r="A83" s="4" t="s">
         <v>176</v>
       </c>
@@ -5111,7 +5103,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:13" ht="28.5">
+    <row r="84" spans="1:13" ht="27.6">
       <c r="A84" s="4" t="s">
         <v>178</v>
       </c>
@@ -5321,7 +5313,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="1:13" ht="28.5">
+    <row r="89" spans="1:13" ht="27.6">
       <c r="A89" s="4" t="s">
         <v>188</v>
       </c>
@@ -5363,7 +5355,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="1:13" ht="28.5">
+    <row r="90" spans="1:13">
       <c r="A90" s="4" t="s">
         <v>190</v>
       </c>
@@ -5447,7 +5439,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="1:13" ht="28.5">
+    <row r="92" spans="1:13" ht="27.6">
       <c r="A92" s="4" t="s">
         <v>194</v>
       </c>
@@ -5580,19 +5572,19 @@
     <mergeCell ref="N1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="K11:K94">
-    <cfRule type="expression" dxfId="33" priority="1">
+    <cfRule type="expression" dxfId="32" priority="1">
       <formula>$K11="Finalizado"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="2">
+    <cfRule type="expression" dxfId="31" priority="2">
       <formula>$K11="En progreso"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="3">
+    <cfRule type="expression" dxfId="30" priority="3">
       <formula>$K11="Validación"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="4">
+    <cfRule type="expression" dxfId="29" priority="4">
       <formula>$K11="Pendiente"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="5">
+    <cfRule type="expression" dxfId="28" priority="5">
       <formula>$K11="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5614,10 +5606,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="51.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.8984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.09765625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
@@ -5628,7 +5620,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.95" customHeight="1">
+    <row r="1" spans="1:11" ht="27.9" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>200</v>
       </c>
@@ -5643,7 +5635,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.5">
+    <row r="2" spans="1:11" ht="16.8">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -5661,7 +5653,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.5">
+    <row r="3" spans="1:11" ht="16.8">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -5679,7 +5671,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5">
+    <row r="4" spans="1:11" ht="16.8">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -5697,7 +5689,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5">
+    <row r="5" spans="1:11" ht="16.8">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -5715,7 +5707,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.5">
+    <row r="6" spans="1:11" ht="16.8">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -5772,7 +5764,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15">
+    <row r="10" spans="1:11">
       <c r="A10" s="4" t="s">
         <v>30</v>
       </c>
@@ -5808,7 +5800,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15">
+    <row r="11" spans="1:11">
       <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
@@ -5844,7 +5836,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15">
+    <row r="12" spans="1:11">
       <c r="A12" s="4" t="s">
         <v>35</v>
       </c>
@@ -5880,7 +5872,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="29.25">
+    <row r="13" spans="1:11">
       <c r="A13" s="4" t="s">
         <v>37</v>
       </c>
@@ -5916,7 +5908,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15">
+    <row r="14" spans="1:11">
       <c r="A14" s="4" t="s">
         <v>39</v>
       </c>
@@ -5952,7 +5944,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15">
+    <row r="15" spans="1:11">
       <c r="A15" s="4" t="s">
         <v>41</v>
       </c>
@@ -5988,7 +5980,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15">
+    <row r="16" spans="1:11">
       <c r="A16" s="4" t="s">
         <v>43</v>
       </c>
@@ -6024,7 +6016,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="29.25">
+    <row r="17" spans="1:11" ht="27.6">
       <c r="A17" s="4" t="s">
         <v>45</v>
       </c>
@@ -6060,7 +6052,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15">
+    <row r="18" spans="1:11">
       <c r="A18" s="4" t="s">
         <v>47</v>
       </c>
@@ -6096,7 +6088,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15">
+    <row r="19" spans="1:11">
       <c r="A19" s="4" t="s">
         <v>49</v>
       </c>
@@ -6132,7 +6124,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="29.25">
+    <row r="20" spans="1:11" ht="27.6">
       <c r="A20" s="4" t="s">
         <v>51</v>
       </c>
@@ -6168,7 +6160,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15">
+    <row r="21" spans="1:11">
       <c r="A21" s="4" t="s">
         <v>53</v>
       </c>
@@ -6214,16 +6206,16 @@
     <mergeCell ref="B5:E5"/>
   </mergeCells>
   <conditionalFormatting sqref="H10:H21">
-    <cfRule type="expression" dxfId="28" priority="1">
+    <cfRule type="expression" dxfId="27" priority="1">
       <formula>$H10="Finalizado"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="2">
+    <cfRule type="expression" dxfId="26" priority="2">
       <formula>$H10="En progreso"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="3">
+    <cfRule type="expression" dxfId="25" priority="3">
       <formula>$H10="Validación"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="4">
+    <cfRule type="expression" dxfId="24" priority="4">
       <formula>$H10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6245,9 +6237,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="25.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.59765625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -6259,7 +6251,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.95" customHeight="1">
+    <row r="1" spans="1:11" ht="27.9" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>222</v>
       </c>
@@ -6274,7 +6266,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.5">
+    <row r="2" spans="1:11" ht="16.8">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -6292,7 +6284,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.5">
+    <row r="3" spans="1:11" ht="16.8">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -6310,7 +6302,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5">
+    <row r="4" spans="1:11" ht="16.8">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -6328,7 +6320,7 @@
         <v>23.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5">
+    <row r="5" spans="1:11" ht="16.8">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -6346,7 +6338,7 @@
         <v>23.5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.5">
+    <row r="6" spans="1:11" ht="16.8">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -6403,7 +6395,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="29.25">
+    <row r="10" spans="1:11" ht="27.6">
       <c r="A10" s="4" t="s">
         <v>56</v>
       </c>
@@ -6439,7 +6431,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="29.25">
+    <row r="11" spans="1:11" ht="27.6">
       <c r="A11" s="4" t="s">
         <v>58</v>
       </c>
@@ -6475,7 +6467,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="29.25">
+    <row r="12" spans="1:11" ht="27.6">
       <c r="A12" s="4" t="s">
         <v>60</v>
       </c>
@@ -6583,7 +6575,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15">
+    <row r="15" spans="1:11">
       <c r="A15" s="4" t="s">
         <v>66</v>
       </c>
@@ -6619,7 +6611,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15">
+    <row r="16" spans="1:11">
       <c r="A16" s="4" t="s">
         <v>68</v>
       </c>
@@ -6655,7 +6647,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15">
+    <row r="17" spans="1:11">
       <c r="A17" s="4" t="s">
         <v>70</v>
       </c>
@@ -6691,7 +6683,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="29.25">
+    <row r="18" spans="1:11" ht="27.6">
       <c r="A18" s="4" t="s">
         <v>72</v>
       </c>
@@ -6727,7 +6719,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15">
+    <row r="19" spans="1:11">
       <c r="A19" s="4" t="s">
         <v>74</v>
       </c>
@@ -6763,7 +6755,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="29.25">
+    <row r="20" spans="1:11" ht="27.6">
       <c r="A20" s="4" t="s">
         <v>76</v>
       </c>
@@ -6799,7 +6791,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="29.25">
+    <row r="21" spans="1:11" ht="27.6">
       <c r="A21" s="4" t="s">
         <v>78</v>
       </c>
@@ -6835,7 +6827,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="29.25">
+    <row r="22" spans="1:11" ht="27.6">
       <c r="A22" s="4" t="s">
         <v>80</v>
       </c>
@@ -6871,7 +6863,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15">
+    <row r="23" spans="1:11">
       <c r="A23" s="4" t="s">
         <v>82</v>
       </c>
@@ -6917,21 +6909,21 @@
     <mergeCell ref="B5:E5"/>
   </mergeCells>
   <conditionalFormatting sqref="F19 F21:F23">
-    <cfRule type="expression" dxfId="24" priority="5">
+    <cfRule type="expression" dxfId="23" priority="5">
       <formula>AND($H19="Finalizado",$F19="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:H23">
-    <cfRule type="expression" dxfId="23" priority="1">
+    <cfRule type="expression" dxfId="22" priority="1">
       <formula>$H10="Finalizado"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="2">
+    <cfRule type="expression" dxfId="21" priority="2">
       <formula>$H10="En progreso"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="3">
+    <cfRule type="expression" dxfId="20" priority="3">
       <formula>$H10="Validación"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="4">
+    <cfRule type="expression" dxfId="19" priority="4">
       <formula>$H10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6953,9 +6945,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="25.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.19921875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -6967,7 +6959,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.95" customHeight="1">
+    <row r="1" spans="1:11" ht="27.9" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>227</v>
       </c>
@@ -6982,7 +6974,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.5">
+    <row r="2" spans="1:11" ht="16.8">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -7000,7 +6992,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.5">
+    <row r="3" spans="1:11" ht="16.8">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -7018,7 +7010,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5">
+    <row r="4" spans="1:11" ht="16.8">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -7036,7 +7028,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5">
+    <row r="5" spans="1:11" ht="16.8">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -7054,7 +7046,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.5">
+    <row r="6" spans="1:11" ht="16.8">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -7111,7 +7103,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15">
+    <row r="10" spans="1:11">
       <c r="A10" s="4" t="s">
         <v>84</v>
       </c>
@@ -7147,7 +7139,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="29.25">
+    <row r="11" spans="1:11" ht="27.6">
       <c r="A11" s="4" t="s">
         <v>86</v>
       </c>
@@ -7183,7 +7175,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15">
+    <row r="12" spans="1:11">
       <c r="A12" s="4" t="s">
         <v>88</v>
       </c>
@@ -7219,7 +7211,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15">
+    <row r="13" spans="1:11">
       <c r="A13" s="4" t="s">
         <v>90</v>
       </c>
@@ -7255,7 +7247,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15">
+    <row r="14" spans="1:11">
       <c r="A14" s="4" t="s">
         <v>92</v>
       </c>
@@ -7327,7 +7319,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="28.5">
+    <row r="16" spans="1:11">
       <c r="A16" s="4" t="s">
         <v>96</v>
       </c>
@@ -7363,7 +7355,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15">
+    <row r="17" spans="1:11">
       <c r="A17" s="4" t="s">
         <v>98</v>
       </c>
@@ -7435,7 +7427,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="28.5">
+    <row r="19" spans="1:11" ht="27.6">
       <c r="A19" s="4" t="s">
         <v>102</v>
       </c>
@@ -7512,7 +7504,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7526,7 +7518,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.95" customHeight="1">
+    <row r="1" spans="1:11" ht="27.9" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>232</v>
       </c>
@@ -7541,7 +7533,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.5">
+    <row r="2" spans="1:11" ht="16.8">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -7559,7 +7551,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.5">
+    <row r="3" spans="1:11" ht="16.8">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -7577,7 +7569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5">
+    <row r="4" spans="1:11" ht="16.8">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -7595,7 +7587,7 @@
         <v>22.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5">
+    <row r="5" spans="1:11" ht="16.8">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -7610,16 +7602,16 @@
       </c>
       <c r="H5" s="2">
         <f>SUM(F10:F19)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="16.5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="16.8">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
       <c r="H6" s="2">
         <f>SUM(G10:G19)</f>
-        <v>22.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -7677,7 +7669,9 @@
       <c r="B10" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D10" s="4" t="s">
         <v>32</v>
       </c>
@@ -7703,7 +7697,9 @@
       <c r="B11" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D11" s="4" t="s">
         <v>32</v>
       </c>
@@ -7729,23 +7725,31 @@
       <c r="B12" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D12" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E12" s="6">
         <v>2</v>
       </c>
-      <c r="F12" s="6"/>
+      <c r="F12" s="6">
+        <v>2</v>
+      </c>
       <c r="G12" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
+        <v>256</v>
+      </c>
+      <c r="I12" s="5">
+        <v>46302</v>
+      </c>
+      <c r="J12" s="5">
+        <v>46304</v>
+      </c>
       <c r="K12" s="4"/>
     </row>
     <row r="13" spans="1:11">
@@ -7755,23 +7759,31 @@
       <c r="B13" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D13" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E13" s="6">
         <v>2</v>
       </c>
-      <c r="F13" s="6"/>
+      <c r="F13" s="6">
+        <v>2</v>
+      </c>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
+        <v>256</v>
+      </c>
+      <c r="I13" s="5">
+        <v>46302</v>
+      </c>
+      <c r="J13" s="5">
+        <v>46304</v>
+      </c>
       <c r="K13" s="4"/>
     </row>
     <row r="14" spans="1:11">
@@ -7781,23 +7793,31 @@
       <c r="B14" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D14" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E14" s="6">
         <v>2</v>
       </c>
-      <c r="F14" s="6"/>
+      <c r="F14" s="6">
+        <v>2</v>
+      </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
+        <v>256</v>
+      </c>
+      <c r="I14" s="5">
+        <v>46302</v>
+      </c>
+      <c r="J14" s="5">
+        <v>46304</v>
+      </c>
       <c r="K14" s="4"/>
     </row>
     <row r="15" spans="1:11">
@@ -7807,23 +7827,31 @@
       <c r="B15" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D15" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E15" s="6">
         <v>2</v>
       </c>
-      <c r="F15" s="6"/>
+      <c r="F15" s="6">
+        <v>2</v>
+      </c>
       <c r="G15" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
+        <v>256</v>
+      </c>
+      <c r="I15" s="5">
+        <v>46302</v>
+      </c>
+      <c r="J15" s="5">
+        <v>46304</v>
+      </c>
       <c r="K15" s="4"/>
     </row>
     <row r="16" spans="1:11">
@@ -7833,26 +7861,34 @@
       <c r="B16" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D16" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E16" s="6">
         <v>2</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="6">
+        <v>2</v>
+      </c>
       <c r="G16" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
+        <v>256</v>
+      </c>
+      <c r="I16" s="5">
+        <v>46302</v>
+      </c>
+      <c r="J16" s="5">
+        <v>46304</v>
+      </c>
       <c r="K16" s="4"/>
     </row>
-    <row r="17" spans="1:11" ht="28.5">
+    <row r="17" spans="1:11" ht="27.6">
       <c r="A17" s="4" t="s">
         <v>118</v>
       </c>
@@ -7878,7 +7914,7 @@
       <c r="J17" s="5"/>
       <c r="K17" s="4"/>
     </row>
-    <row r="18" spans="1:11" ht="28.5">
+    <row r="18" spans="1:11" ht="27.6">
       <c r="A18" s="4" t="s">
         <v>120</v>
       </c>
@@ -7904,7 +7940,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="4"/>
     </row>
-    <row r="19" spans="1:11" ht="28.5">
+    <row r="19" spans="1:11" ht="27.6">
       <c r="A19" s="4" t="s">
         <v>122</v>
       </c>
@@ -7939,7 +7975,7 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:F19">
+  <conditionalFormatting sqref="F10:F11 F17:F19">
     <cfRule type="expression" dxfId="14" priority="5">
       <formula>AND($H10="Finalizado",$F10="")</formula>
     </cfRule>
@@ -7976,9 +8012,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.59765625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -7990,7 +8026,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.95" customHeight="1">
+    <row r="1" spans="1:11" ht="27.9" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>236</v>
       </c>
@@ -8005,7 +8041,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.5">
+    <row r="2" spans="1:11" ht="16.8">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -8023,7 +8059,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.5">
+    <row r="3" spans="1:11" ht="16.8">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -8041,7 +8077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5">
+    <row r="4" spans="1:11" ht="16.8">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -8059,7 +8095,7 @@
         <v>24.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5">
+    <row r="5" spans="1:11" ht="16.8">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -8077,7 +8113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.5">
+    <row r="6" spans="1:11" ht="16.8">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -8134,14 +8170,16 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="28.5">
+    <row r="10" spans="1:11" ht="27.6">
       <c r="A10" s="4" t="s">
         <v>124</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D10" s="4" t="s">
         <v>32</v>
       </c>
@@ -8167,7 +8205,9 @@
       <c r="B11" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D11" s="4" t="s">
         <v>32</v>
       </c>
@@ -8186,14 +8226,16 @@
       <c r="J11" s="5"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11" ht="28.5">
+    <row r="12" spans="1:11" ht="27.6">
       <c r="A12" s="4" t="s">
         <v>128</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D12" s="4" t="s">
         <v>32</v>
       </c>
@@ -8219,7 +8261,9 @@
       <c r="B13" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D13" s="4" t="s">
         <v>32</v>
       </c>
@@ -8238,14 +8282,16 @@
       <c r="J13" s="5"/>
       <c r="K13" s="4"/>
     </row>
-    <row r="14" spans="1:11" ht="28.5">
+    <row r="14" spans="1:11" ht="27.6">
       <c r="A14" s="4" t="s">
         <v>132</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D14" s="4" t="s">
         <v>32</v>
       </c>
@@ -8271,7 +8317,9 @@
       <c r="B15" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D15" s="4" t="s">
         <v>32</v>
       </c>
@@ -8297,7 +8345,9 @@
       <c r="B16" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="D16" s="4" t="s">
         <v>32</v>
       </c>
@@ -8323,7 +8373,9 @@
       <c r="B17" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D17" s="4" t="s">
         <v>32</v>
       </c>
@@ -8349,7 +8401,9 @@
       <c r="B18" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D18" s="4" t="s">
         <v>32</v>
       </c>
@@ -8375,7 +8429,9 @@
       <c r="B19" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D19" s="4" t="s">
         <v>32</v>
       </c>
@@ -8401,7 +8457,9 @@
       <c r="B20" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D20" s="4" t="s">
         <v>32</v>
       </c>
@@ -8427,7 +8485,9 @@
       <c r="B21" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D21" s="4" t="s">
         <v>32</v>
       </c>
@@ -8453,7 +8513,9 @@
       <c r="B22" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="4" t="s">
+        <v>254</v>
+      </c>
       <c r="D22" s="4" t="s">
         <v>32</v>
       </c>
@@ -8479,7 +8541,9 @@
       <c r="B23" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D23" s="4" t="s">
         <v>32</v>
       </c>
@@ -8505,7 +8569,9 @@
       <c r="B24" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D24" s="4" t="s">
         <v>32</v>
       </c>
@@ -8531,7 +8597,9 @@
       <c r="B25" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D25" s="4" t="s">
         <v>32</v>
       </c>
@@ -8550,14 +8618,16 @@
       <c r="J25" s="5"/>
       <c r="K25" s="4"/>
     </row>
-    <row r="26" spans="1:11" ht="28.5">
+    <row r="26" spans="1:11" ht="27.6">
       <c r="A26" s="4" t="s">
         <v>156</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C26" s="4"/>
+      <c r="C26" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D26" s="4" t="s">
         <v>55</v>
       </c>
@@ -8576,14 +8646,16 @@
       <c r="J26" s="5"/>
       <c r="K26" s="4"/>
     </row>
-    <row r="27" spans="1:11" ht="28.5">
+    <row r="27" spans="1:11" ht="27.6">
       <c r="A27" s="4" t="s">
         <v>158</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="D27" s="4" t="s">
         <v>32</v>
       </c>
@@ -8648,9 +8720,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.59765625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -8662,7 +8734,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.95" customHeight="1">
+    <row r="1" spans="1:11" ht="27.9" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>241</v>
       </c>
@@ -8677,7 +8749,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.5">
+    <row r="2" spans="1:11" ht="16.8">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -8695,7 +8767,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.5">
+    <row r="3" spans="1:11" ht="16.8">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -8713,7 +8785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5">
+    <row r="4" spans="1:11" ht="16.8">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -8731,7 +8803,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5">
+    <row r="5" spans="1:11" ht="16.8">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -8749,7 +8821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.5">
+    <row r="6" spans="1:11" ht="16.8">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -8858,7 +8930,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11" ht="28.5">
+    <row r="12" spans="1:11">
       <c r="A12" s="4" t="s">
         <v>164</v>
       </c>
@@ -8962,7 +9034,7 @@
       <c r="J15" s="5"/>
       <c r="K15" s="4"/>
     </row>
-    <row r="16" spans="1:11" ht="28.5">
+    <row r="16" spans="1:11" ht="27.6">
       <c r="A16" s="4" t="s">
         <v>172</v>
       </c>
@@ -9014,7 +9086,7 @@
       <c r="J17" s="5"/>
       <c r="K17" s="4"/>
     </row>
-    <row r="18" spans="1:11" ht="28.5">
+    <row r="18" spans="1:11" ht="27.6">
       <c r="A18" s="4" t="s">
         <v>176</v>
       </c>
@@ -9040,7 +9112,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="4"/>
     </row>
-    <row r="19" spans="1:11" ht="28.5">
+    <row r="19" spans="1:11" ht="27.6">
       <c r="A19" s="4" t="s">
         <v>178</v>
       </c>
@@ -9170,7 +9242,7 @@
       <c r="J23" s="5"/>
       <c r="K23" s="4"/>
     </row>
-    <row r="24" spans="1:11" ht="28.5">
+    <row r="24" spans="1:11" ht="27.6">
       <c r="A24" s="4" t="s">
         <v>188</v>
       </c>
@@ -9196,7 +9268,7 @@
       <c r="J24" s="5"/>
       <c r="K24" s="4"/>
     </row>
-    <row r="25" spans="1:11" ht="28.5">
+    <row r="25" spans="1:11" ht="27.6">
       <c r="A25" s="4" t="s">
         <v>190</v>
       </c>
@@ -9248,7 +9320,7 @@
       <c r="J26" s="5"/>
       <c r="K26" s="4"/>
     </row>
-    <row r="27" spans="1:11" ht="28.5">
+    <row r="27" spans="1:11" ht="27.6">
       <c r="A27" s="4" t="s">
         <v>194</v>
       </c>

</xml_diff>

<commit_message>
Sprint 5 - Integración técnica y validación de CAPEX/OPEX
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3FEFF9-139A-4CA3-BD5A-4A6B05AAB566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75958461-B419-4532-B9A7-1F3FE4C75EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -1748,28 +1748,28 @@
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(K11:K94,"Finalizado")</f>
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="2">
         <f>COUNTIF(K11:K94,"Pendiente")</f>
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="2">
         <f>SUM(I11:I94)</f>
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="2">
         <f>SUM(J11:J94)</f>
-        <v>61.5</v>
+        <v>52.5</v>
       </c>
       <c r="N4" t="s">
         <v>12</v>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="Q7">
         <f>COUNTIFS(D11:D94,5,K11:K94,"Finalizado")</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -3546,7 +3546,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:13" ht="15">
       <c r="A47" s="4" t="s">
         <v>104</v>
       </c>
@@ -3588,7 +3588,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:13" ht="15">
       <c r="A48" s="4" t="s">
         <v>106</v>
       </c>
@@ -3840,7 +3840,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="28.5">
+    <row r="54" spans="1:13" ht="29.25">
       <c r="A54" s="4" t="s">
         <v>118</v>
       </c>
@@ -3882,7 +3882,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="28.5">
+    <row r="55" spans="1:13" ht="29.25">
       <c r="A55" s="4" t="s">
         <v>120</v>
       </c>
@@ -3924,7 +3924,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="28.5">
+    <row r="56" spans="1:13" ht="29.25">
       <c r="A56" s="4" t="s">
         <v>122</v>
       </c>
@@ -3987,17 +3987,17 @@
       <c r="H57" s="6">
         <v>1</v>
       </c>
-      <c r="I57" s="6" t="str">
+      <c r="I57" s="6">
         <f>IF('Sprint 5'!F10="","",'Sprint 5'!F10)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J57" s="6">
         <f>'Sprint 5'!G10</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K57" s="4" t="str">
         <f>'Sprint 5'!H10</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L57" s="4" t="str">
         <f>IF('Sprint 5'!C10="","",'Sprint 5'!C10)</f>
@@ -4029,17 +4029,17 @@
       <c r="H58" s="6">
         <v>1</v>
       </c>
-      <c r="I58" s="6" t="str">
+      <c r="I58" s="6">
         <f>IF('Sprint 5'!F11="","",'Sprint 5'!F11)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J58" s="6">
         <f>'Sprint 5'!G11</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K58" s="4" t="str">
         <f>'Sprint 5'!H11</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L58" s="4" t="str">
         <f>IF('Sprint 5'!C11="","",'Sprint 5'!C11)</f>
@@ -4071,17 +4071,17 @@
       <c r="H59" s="6">
         <v>1</v>
       </c>
-      <c r="I59" s="6" t="str">
+      <c r="I59" s="6">
         <f>IF('Sprint 5'!F12="","",'Sprint 5'!F12)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J59" s="6">
         <f>'Sprint 5'!G12</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K59" s="4" t="str">
         <f>'Sprint 5'!H12</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L59" s="4" t="str">
         <f>IF('Sprint 5'!C12="","",'Sprint 5'!C12)</f>
@@ -4092,7 +4092,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="1:13">
+    <row r="60" spans="1:13" ht="15">
       <c r="A60" s="4" t="s">
         <v>130</v>
       </c>
@@ -4113,17 +4113,17 @@
       <c r="H60" s="6">
         <v>2</v>
       </c>
-      <c r="I60" s="6" t="str">
+      <c r="I60" s="6">
         <f>IF('Sprint 5'!F13="","",'Sprint 5'!F13)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J60" s="6">
         <f>'Sprint 5'!G13</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K60" s="4" t="str">
         <f>'Sprint 5'!H13</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L60" s="4" t="str">
         <f>IF('Sprint 5'!C13="","",'Sprint 5'!C13)</f>
@@ -4134,7 +4134,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:13">
+    <row r="61" spans="1:13" ht="15">
       <c r="A61" s="4" t="s">
         <v>132</v>
       </c>
@@ -4155,17 +4155,17 @@
       <c r="H61" s="6">
         <v>1</v>
       </c>
-      <c r="I61" s="6" t="str">
+      <c r="I61" s="6">
         <f>IF('Sprint 5'!F14="","",'Sprint 5'!F14)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J61" s="6">
         <f>'Sprint 5'!G14</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K61" s="4" t="str">
         <f>'Sprint 5'!H14</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L61" s="4" t="str">
         <f>IF('Sprint 5'!C14="","",'Sprint 5'!C14)</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:13">
+    <row r="62" spans="1:13" ht="15">
       <c r="A62" s="4" t="s">
         <v>134</v>
       </c>
@@ -4197,17 +4197,17 @@
       <c r="H62" s="6">
         <v>1.5</v>
       </c>
-      <c r="I62" s="6" t="str">
+      <c r="I62" s="6">
         <f>IF('Sprint 5'!F15="","",'Sprint 5'!F15)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J62" s="6">
         <f>'Sprint 5'!G15</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K62" s="4" t="str">
         <f>'Sprint 5'!H15</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L62" s="4" t="str">
         <f>IF('Sprint 5'!C15="","",'Sprint 5'!C15)</f>
@@ -4218,7 +4218,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="1:13">
+    <row r="63" spans="1:13" ht="15">
       <c r="A63" s="4" t="s">
         <v>136</v>
       </c>
@@ -4239,17 +4239,17 @@
       <c r="H63" s="6">
         <v>1.5</v>
       </c>
-      <c r="I63" s="6" t="str">
+      <c r="I63" s="6">
         <f>IF('Sprint 5'!F16="","",'Sprint 5'!F16)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J63" s="6">
         <f>'Sprint 5'!G16</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K63" s="4" t="str">
         <f>'Sprint 5'!H16</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L63" s="4" t="str">
         <f>IF('Sprint 5'!C16="","",'Sprint 5'!C16)</f>
@@ -8127,7 +8127,7 @@
       </c>
       <c r="H3" s="2">
         <f>COUNTIF(H10:H27,"Finalizado")</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="16.5">
@@ -8163,7 +8163,7 @@
       </c>
       <c r="H5" s="2">
         <f>SUM(F10:F27)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="16.5">
@@ -8172,7 +8172,7 @@
       </c>
       <c r="H6" s="2">
         <f>SUM(G10:G27)</f>
-        <v>24.5</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -8223,7 +8223,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="28.5">
+    <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="4" t="s">
         <v>124</v>
       </c>
@@ -8239,19 +8239,25 @@
       <c r="E10" s="6">
         <v>1</v>
       </c>
-      <c r="F10" s="6"/>
+      <c r="F10" s="6">
+        <v>1</v>
+      </c>
       <c r="G10" s="6">
         <f t="shared" ref="G10:G27" si="0">IF(H10="Finalizado",0,MAX(E10-IF(F10="",0,F10),0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I10" s="5">
+        <v>46305</v>
+      </c>
+      <c r="J10" s="5">
+        <v>46309</v>
+      </c>
       <c r="K10" s="4"/>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" ht="15">
       <c r="A11" s="4" t="s">
         <v>126</v>
       </c>
@@ -8267,19 +8273,25 @@
       <c r="E11" s="6">
         <v>1</v>
       </c>
-      <c r="F11" s="6"/>
+      <c r="F11" s="6">
+        <v>1</v>
+      </c>
       <c r="G11" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I11" s="5">
+        <v>46305</v>
+      </c>
+      <c r="J11" s="5">
+        <v>46309</v>
+      </c>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11" ht="28.5">
+    <row r="12" spans="1:11" ht="29.25">
       <c r="A12" s="4" t="s">
         <v>128</v>
       </c>
@@ -8295,19 +8307,25 @@
       <c r="E12" s="6">
         <v>1</v>
       </c>
-      <c r="F12" s="6"/>
+      <c r="F12" s="6">
+        <v>1</v>
+      </c>
       <c r="G12" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I12" s="5">
+        <v>46305</v>
+      </c>
+      <c r="J12" s="5">
+        <v>46309</v>
+      </c>
       <c r="K12" s="4"/>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" ht="15">
       <c r="A13" s="4" t="s">
         <v>130</v>
       </c>
@@ -8323,19 +8341,25 @@
       <c r="E13" s="6">
         <v>2</v>
       </c>
-      <c r="F13" s="6"/>
+      <c r="F13" s="6">
+        <v>2</v>
+      </c>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I13" s="5">
+        <v>46305</v>
+      </c>
+      <c r="J13" s="5">
+        <v>46309</v>
+      </c>
       <c r="K13" s="4"/>
     </row>
-    <row r="14" spans="1:11" ht="28.5">
+    <row r="14" spans="1:11" ht="29.25">
       <c r="A14" s="4" t="s">
         <v>132</v>
       </c>
@@ -8351,19 +8375,25 @@
       <c r="E14" s="6">
         <v>1</v>
       </c>
-      <c r="F14" s="6"/>
+      <c r="F14" s="6">
+        <v>1</v>
+      </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I14" s="5">
+        <v>46305</v>
+      </c>
+      <c r="J14" s="5">
+        <v>46309</v>
+      </c>
       <c r="K14" s="4"/>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" ht="15">
       <c r="A15" s="4" t="s">
         <v>134</v>
       </c>
@@ -8379,19 +8409,25 @@
       <c r="E15" s="6">
         <v>1.5</v>
       </c>
-      <c r="F15" s="6"/>
+      <c r="F15" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G15" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I15" s="5">
+        <v>46305</v>
+      </c>
+      <c r="J15" s="5">
+        <v>46309</v>
+      </c>
       <c r="K15" s="4"/>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" ht="15">
       <c r="A16" s="4" t="s">
         <v>136</v>
       </c>
@@ -8407,16 +8443,22 @@
       <c r="E16" s="6">
         <v>1.5</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G16" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
+        <v>220</v>
+      </c>
+      <c r="I16" s="5">
+        <v>46305</v>
+      </c>
+      <c r="J16" s="5">
+        <v>46309</v>
+      </c>
       <c r="K16" s="4"/>
     </row>
     <row r="17" spans="1:11">
@@ -8736,9 +8778,9 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:F27">
+  <conditionalFormatting sqref="F17:F27">
     <cfRule type="expression" dxfId="9" priority="5">
-      <formula>AND($H10="Finalizado",$F10="")</formula>
+      <formula>AND($H17="Finalizado",$F17="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:H27">

</xml_diff>

<commit_message>
Tercera entrega finalizada - Sprints 4 y 5
</commit_message>
<xml_diff>
--- a/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
+++ b/Docs/Capstone_FWA_SCRUM_Backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Barrios\Desktop\capstone-fwa-rural-main (2)\capstone-fwa-rural-main\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USUARIO\Desktop\Capstone-FWA\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B708FCC6-DCA4-45AB-B1AF-B239AE4B132B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80DB297-31E6-404F-BE1C-E684FC8A09BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="256">
   <si>
     <t>Product Backlog – Capstone 5G FWA Rural</t>
   </si>
@@ -1640,15 +1640,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q94"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.69921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.8984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="19.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
@@ -1661,7 +1661,7 @@
     <col min="17" max="17" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="27.9" customHeight="1">
+    <row r="1" spans="1:17" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1684,7 +1684,7 @@
       <c r="P1" s="9"/>
       <c r="Q1" s="9"/>
     </row>
-    <row r="2" spans="1:17" ht="33.9" customHeight="1">
+    <row r="2" spans="1:17" ht="33.950000000000003" customHeight="1">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1728,7 +1728,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="16.8">
+    <row r="4" spans="1:17" ht="16.5">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -1748,28 +1748,28 @@
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(K11:K94,"Finalizado")</f>
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="2">
         <f>COUNTIF(K11:K94,"Pendiente")</f>
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="2">
         <f>SUM(I11:I94)</f>
-        <v>92</v>
+        <v>99.5</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="2">
         <f>SUM(J11:J94)</f>
-        <v>44.5</v>
+        <v>37</v>
       </c>
       <c r="N4" t="s">
         <v>12</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" ht="15">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="Q7">
         <f>COUNTIFS(D11:D94,5,K11:K94,"Finalizado")</f>
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1859,7 +1859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="41.4">
+    <row r="10" spans="1:17" ht="45">
       <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
@@ -1900,7 +1900,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" ht="15">
       <c r="A11" s="4" t="s">
         <v>30</v>
       </c>
@@ -1945,7 +1945,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" ht="15">
       <c r="A12" s="4" t="s">
         <v>33</v>
       </c>
@@ -1990,7 +1990,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="27.6">
+    <row r="13" spans="1:17" ht="29.25">
       <c r="A13" s="4" t="s">
         <v>35</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="27.6">
+    <row r="14" spans="1:17" ht="29.25">
       <c r="A14" s="4" t="s">
         <v>37</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" ht="15">
       <c r="A15" s="4" t="s">
         <v>39</v>
       </c>
@@ -2125,7 +2125,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" ht="15">
       <c r="A16" s="4" t="s">
         <v>41</v>
       </c>
@@ -2170,7 +2170,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" ht="15">
       <c r="A17" s="4" t="s">
         <v>43</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="27.6">
+    <row r="18" spans="1:13" ht="29.25">
       <c r="A18" s="4" t="s">
         <v>45</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" ht="15">
       <c r="A19" s="4" t="s">
         <v>47</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" ht="15">
       <c r="A20" s="4" t="s">
         <v>49</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="27.6">
+    <row r="21" spans="1:13" ht="29.25">
       <c r="A21" s="4" t="s">
         <v>51</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" ht="15">
       <c r="A22" s="4" t="s">
         <v>53</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="27.6">
+    <row r="23" spans="1:13" ht="29.25">
       <c r="A23" s="4" t="s">
         <v>56</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="27.6">
+    <row r="24" spans="1:13" ht="29.25">
       <c r="A24" s="4" t="s">
         <v>58</v>
       </c>
@@ -2534,7 +2534,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="27.6">
+    <row r="25" spans="1:13" ht="29.25">
       <c r="A25" s="4" t="s">
         <v>60</v>
       </c>
@@ -2580,7 +2580,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" ht="15">
       <c r="A26" s="4" t="s">
         <v>62</v>
       </c>
@@ -2626,7 +2626,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" ht="15">
       <c r="A27" s="4" t="s">
         <v>64</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" ht="15">
       <c r="A28" s="4" t="s">
         <v>66</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" ht="15">
       <c r="A29" s="4" t="s">
         <v>68</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" ht="15">
       <c r="A30" s="4" t="s">
         <v>70</v>
       </c>
@@ -2810,7 +2810,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="27.6">
+    <row r="31" spans="1:13" ht="29.25">
       <c r="A31" s="4" t="s">
         <v>72</v>
       </c>
@@ -2856,7 +2856,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" ht="15">
       <c r="A32" s="4" t="s">
         <v>74</v>
       </c>
@@ -2902,7 +2902,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" ht="29.25">
       <c r="A33" s="4" t="s">
         <v>76</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="27.6">
+    <row r="34" spans="1:13" ht="29.25">
       <c r="A34" s="4" t="s">
         <v>78</v>
       </c>
@@ -2994,7 +2994,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" ht="29.25">
       <c r="A35" s="4" t="s">
         <v>80</v>
       </c>
@@ -3040,7 +3040,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:13" ht="15">
       <c r="A36" s="4" t="s">
         <v>82</v>
       </c>
@@ -3086,7 +3086,7 @@
         <v>Realizado con éxito</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" ht="15">
       <c r="A37" s="4" t="s">
         <v>84</v>
       </c>
@@ -3132,7 +3132,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="27.6">
+    <row r="38" spans="1:13" ht="29.25">
       <c r="A38" s="4" t="s">
         <v>86</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:13" ht="15">
       <c r="A39" s="4" t="s">
         <v>88</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:13" ht="15">
       <c r="A40" s="4" t="s">
         <v>90</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:13" ht="15">
       <c r="A41" s="4" t="s">
         <v>92</v>
       </c>
@@ -3316,7 +3316,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="42" spans="1:13">
+    <row r="42" spans="1:13" ht="15">
       <c r="A42" s="4" t="s">
         <v>94</v>
       </c>
@@ -3362,7 +3362,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="43" spans="1:13">
+    <row r="43" spans="1:13" ht="15">
       <c r="A43" s="4" t="s">
         <v>96</v>
       </c>
@@ -3408,7 +3408,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" ht="15">
       <c r="A44" s="4" t="s">
         <v>98</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="45" spans="1:13">
+    <row r="45" spans="1:13" ht="15">
       <c r="A45" s="4" t="s">
         <v>100</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="46" spans="1:13">
+    <row r="46" spans="1:13" ht="15">
       <c r="A46" s="4" t="s">
         <v>102</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:13" ht="15">
       <c r="A47" s="4" t="s">
         <v>104</v>
       </c>
@@ -3588,7 +3588,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:13" ht="15">
       <c r="A48" s="4" t="s">
         <v>106</v>
       </c>
@@ -3630,7 +3630,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="49" spans="1:13">
+    <row r="49" spans="1:13" ht="15">
       <c r="A49" s="4" t="s">
         <v>108</v>
       </c>
@@ -3672,7 +3672,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="50" spans="1:13">
+    <row r="50" spans="1:13" ht="15">
       <c r="A50" s="4" t="s">
         <v>110</v>
       </c>
@@ -3714,7 +3714,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="51" spans="1:13">
+    <row r="51" spans="1:13" ht="15">
       <c r="A51" s="4" t="s">
         <v>112</v>
       </c>
@@ -3756,7 +3756,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="52" spans="1:13">
+    <row r="52" spans="1:13" ht="15">
       <c r="A52" s="4" t="s">
         <v>114</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="53" spans="1:13">
+    <row r="53" spans="1:13" ht="15">
       <c r="A53" s="4" t="s">
         <v>116</v>
       </c>
@@ -3840,7 +3840,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="27.6">
+    <row r="54" spans="1:13" ht="29.25">
       <c r="A54" s="4" t="s">
         <v>118</v>
       </c>
@@ -3882,7 +3882,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="27.6">
+    <row r="55" spans="1:13" ht="29.25">
       <c r="A55" s="4" t="s">
         <v>120</v>
       </c>
@@ -3924,7 +3924,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="27.6">
+    <row r="56" spans="1:13" ht="29.25">
       <c r="A56" s="4" t="s">
         <v>122</v>
       </c>
@@ -3966,7 +3966,7 @@
         <v>Terminado con éxito</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="27.6">
+    <row r="57" spans="1:13" ht="29.25">
       <c r="A57" s="4" t="s">
         <v>124</v>
       </c>
@@ -4005,10 +4005,10 @@
       </c>
       <c r="M57" s="4" t="str">
         <f>IF('Sprint 5'!K10="","",'Sprint 5'!K10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" ht="15">
       <c r="A58" s="4" t="s">
         <v>126</v>
       </c>
@@ -4047,10 +4047,10 @@
       </c>
       <c r="M58" s="4" t="str">
         <f>IF('Sprint 5'!K11="","",'Sprint 5'!K11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="1:13" ht="27.6">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" ht="29.25">
       <c r="A59" s="4" t="s">
         <v>128</v>
       </c>
@@ -4089,10 +4089,10 @@
       </c>
       <c r="M59" s="4" t="str">
         <f>IF('Sprint 5'!K12="","",'Sprint 5'!K12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" ht="15">
       <c r="A60" s="4" t="s">
         <v>130</v>
       </c>
@@ -4131,10 +4131,10 @@
       </c>
       <c r="M60" s="4" t="str">
         <f>IF('Sprint 5'!K13="","",'Sprint 5'!K13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" ht="15">
       <c r="A61" s="4" t="s">
         <v>132</v>
       </c>
@@ -4173,10 +4173,10 @@
       </c>
       <c r="M61" s="4" t="str">
         <f>IF('Sprint 5'!K14="","",'Sprint 5'!K14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" ht="15">
       <c r="A62" s="4" t="s">
         <v>134</v>
       </c>
@@ -4215,10 +4215,10 @@
       </c>
       <c r="M62" s="4" t="str">
         <f>IF('Sprint 5'!K15="","",'Sprint 5'!K15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" ht="15">
       <c r="A63" s="4" t="s">
         <v>136</v>
       </c>
@@ -4257,10 +4257,10 @@
       </c>
       <c r="M63" s="4" t="str">
         <f>IF('Sprint 5'!K16="","",'Sprint 5'!K16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" ht="15">
       <c r="A64" s="4" t="s">
         <v>138</v>
       </c>
@@ -4299,10 +4299,10 @@
       </c>
       <c r="M64" s="4" t="str">
         <f>IF('Sprint 5'!K17="","",'Sprint 5'!K17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" ht="15">
       <c r="A65" s="4" t="s">
         <v>140</v>
       </c>
@@ -4341,10 +4341,10 @@
       </c>
       <c r="M65" s="4" t="str">
         <f>IF('Sprint 5'!K18="","",'Sprint 5'!K18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" ht="15">
       <c r="A66" s="4" t="s">
         <v>142</v>
       </c>
@@ -4383,10 +4383,10 @@
       </c>
       <c r="M66" s="4" t="str">
         <f>IF('Sprint 5'!K19="","",'Sprint 5'!K19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" ht="15">
       <c r="A67" s="4" t="s">
         <v>144</v>
       </c>
@@ -4425,10 +4425,10 @@
       </c>
       <c r="M67" s="4" t="str">
         <f>IF('Sprint 5'!K20="","",'Sprint 5'!K20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" ht="15">
       <c r="A68" s="4" t="s">
         <v>146</v>
       </c>
@@ -4467,10 +4467,10 @@
       </c>
       <c r="M68" s="4" t="str">
         <f>IF('Sprint 5'!K21="","",'Sprint 5'!K21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" ht="15">
       <c r="A69" s="4" t="s">
         <v>148</v>
       </c>
@@ -4509,10 +4509,10 @@
       </c>
       <c r="M69" s="4" t="str">
         <f>IF('Sprint 5'!K22="","",'Sprint 5'!K22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" ht="15">
       <c r="A70" s="4" t="s">
         <v>150</v>
       </c>
@@ -4533,17 +4533,17 @@
       <c r="H70" s="6">
         <v>1.5</v>
       </c>
-      <c r="I70" s="6" t="str">
+      <c r="I70" s="6">
         <f>IF('Sprint 5'!F23="","",'Sprint 5'!F23)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J70" s="6">
         <f>'Sprint 5'!G23</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K70" s="4" t="str">
         <f>'Sprint 5'!H23</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L70" s="4" t="str">
         <f>IF('Sprint 5'!C23="","",'Sprint 5'!C23)</f>
@@ -4551,10 +4551,10 @@
       </c>
       <c r="M70" s="4" t="str">
         <f>IF('Sprint 5'!K23="","",'Sprint 5'!K23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" ht="15">
       <c r="A71" s="4" t="s">
         <v>152</v>
       </c>
@@ -4575,17 +4575,17 @@
       <c r="H71" s="6">
         <v>1.5</v>
       </c>
-      <c r="I71" s="6" t="str">
+      <c r="I71" s="6">
         <f>IF('Sprint 5'!F24="","",'Sprint 5'!F24)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J71" s="6">
         <f>'Sprint 5'!G24</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K71" s="4" t="str">
         <f>'Sprint 5'!H24</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L71" s="4" t="str">
         <f>IF('Sprint 5'!C24="","",'Sprint 5'!C24)</f>
@@ -4593,10 +4593,10 @@
       </c>
       <c r="M71" s="4" t="str">
         <f>IF('Sprint 5'!K24="","",'Sprint 5'!K24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" ht="15">
       <c r="A72" s="4" t="s">
         <v>154</v>
       </c>
@@ -4617,17 +4617,17 @@
       <c r="H72" s="6">
         <v>1.5</v>
       </c>
-      <c r="I72" s="6" t="str">
+      <c r="I72" s="6">
         <f>IF('Sprint 5'!F25="","",'Sprint 5'!F25)</f>
-        <v/>
+        <v>1.5</v>
       </c>
       <c r="J72" s="6">
         <f>'Sprint 5'!G25</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="K72" s="4" t="str">
         <f>'Sprint 5'!H25</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L72" s="4" t="str">
         <f>IF('Sprint 5'!C25="","",'Sprint 5'!C25)</f>
@@ -4635,10 +4635,10 @@
       </c>
       <c r="M72" s="4" t="str">
         <f>IF('Sprint 5'!K25="","",'Sprint 5'!K25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" spans="1:13">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" ht="15">
       <c r="A73" s="4" t="s">
         <v>156</v>
       </c>
@@ -4659,17 +4659,17 @@
       <c r="H73" s="6">
         <v>1</v>
       </c>
-      <c r="I73" s="6" t="str">
+      <c r="I73" s="6">
         <f>IF('Sprint 5'!F26="","",'Sprint 5'!F26)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J73" s="6">
         <f>'Sprint 5'!G26</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K73" s="4" t="str">
         <f>'Sprint 5'!H26</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L73" s="4" t="str">
         <f>IF('Sprint 5'!C26="","",'Sprint 5'!C26)</f>
@@ -4677,10 +4677,10 @@
       </c>
       <c r="M73" s="4" t="str">
         <f>IF('Sprint 5'!K26="","",'Sprint 5'!K26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="1:13" ht="27.6">
+        <v>Realizado con éxito</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" ht="29.25">
       <c r="A74" s="4" t="s">
         <v>158</v>
       </c>
@@ -4701,17 +4701,17 @@
       <c r="H74" s="6">
         <v>2</v>
       </c>
-      <c r="I74" s="6" t="str">
+      <c r="I74" s="6">
         <f>IF('Sprint 5'!F27="","",'Sprint 5'!F27)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J74" s="6">
         <f>'Sprint 5'!G27</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K74" s="4" t="str">
         <f>'Sprint 5'!H27</f>
-        <v>Pendiente</v>
+        <v>Finalizado</v>
       </c>
       <c r="L74" s="4" t="str">
         <f>IF('Sprint 5'!C27="","",'Sprint 5'!C27)</f>
@@ -4719,7 +4719,7 @@
       </c>
       <c r="M74" s="4" t="str">
         <f>IF('Sprint 5'!K27="","",'Sprint 5'!K27)</f>
-        <v/>
+        <v>Realizado con éxito</v>
       </c>
     </row>
     <row r="75" spans="1:13">
@@ -4974,7 +4974,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:13" ht="27.6">
+    <row r="81" spans="1:13" ht="28.5">
       <c r="A81" s="4" t="s">
         <v>172</v>
       </c>
@@ -5058,7 +5058,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:13" ht="27.6">
+    <row r="83" spans="1:13" ht="28.5">
       <c r="A83" s="4" t="s">
         <v>176</v>
       </c>
@@ -5100,7 +5100,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:13" ht="27.6">
+    <row r="84" spans="1:13" ht="28.5">
       <c r="A84" s="4" t="s">
         <v>178</v>
       </c>
@@ -5310,7 +5310,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="1:13" ht="27.6">
+    <row r="89" spans="1:13" ht="28.5">
       <c r="A89" s="4" t="s">
         <v>188</v>
       </c>
@@ -5352,7 +5352,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="1:13">
+    <row r="90" spans="1:13" ht="28.5">
       <c r="A90" s="4" t="s">
         <v>190</v>
       </c>
@@ -5436,7 +5436,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="1:13" ht="27.6">
+    <row r="92" spans="1:13" ht="28.5">
       <c r="A92" s="4" t="s">
         <v>194</v>
       </c>
@@ -5603,10 +5603,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="22.8984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="51.09765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
@@ -5617,7 +5617,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>200</v>
       </c>
@@ -5632,7 +5632,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -5650,7 +5650,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -5668,7 +5668,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -5686,7 +5686,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -5704,7 +5704,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -5761,7 +5761,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" ht="15">
       <c r="A10" s="4" t="s">
         <v>30</v>
       </c>
@@ -5797,7 +5797,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" ht="15">
       <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
@@ -5833,7 +5833,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" ht="15">
       <c r="A12" s="4" t="s">
         <v>35</v>
       </c>
@@ -5869,7 +5869,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" ht="29.25">
       <c r="A13" s="4" t="s">
         <v>37</v>
       </c>
@@ -5905,7 +5905,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" ht="15">
       <c r="A14" s="4" t="s">
         <v>39</v>
       </c>
@@ -5941,7 +5941,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" ht="15">
       <c r="A15" s="4" t="s">
         <v>41</v>
       </c>
@@ -5977,7 +5977,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" ht="15">
       <c r="A16" s="4" t="s">
         <v>43</v>
       </c>
@@ -6013,7 +6013,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="27.6">
+    <row r="17" spans="1:11" ht="29.25">
       <c r="A17" s="4" t="s">
         <v>45</v>
       </c>
@@ -6049,7 +6049,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" ht="15">
       <c r="A18" s="4" t="s">
         <v>47</v>
       </c>
@@ -6085,7 +6085,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" ht="15">
       <c r="A19" s="4" t="s">
         <v>49</v>
       </c>
@@ -6121,7 +6121,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="27.6">
+    <row r="20" spans="1:11" ht="29.25">
       <c r="A20" s="4" t="s">
         <v>51</v>
       </c>
@@ -6157,7 +6157,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" ht="15">
       <c r="A21" s="4" t="s">
         <v>53</v>
       </c>
@@ -6234,9 +6234,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="25.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -6248,7 +6248,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>222</v>
       </c>
@@ -6263,7 +6263,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -6281,7 +6281,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -6299,7 +6299,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -6317,7 +6317,7 @@
         <v>23.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -6335,7 +6335,7 @@
         <v>23.5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -6392,7 +6392,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="27.6">
+    <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="4" t="s">
         <v>56</v>
       </c>
@@ -6428,7 +6428,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="27.6">
+    <row r="11" spans="1:11" ht="29.25">
       <c r="A11" s="4" t="s">
         <v>58</v>
       </c>
@@ -6464,7 +6464,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="27.6">
+    <row r="12" spans="1:11" ht="29.25">
       <c r="A12" s="4" t="s">
         <v>60</v>
       </c>
@@ -6572,7 +6572,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" ht="15">
       <c r="A15" s="4" t="s">
         <v>66</v>
       </c>
@@ -6608,7 +6608,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" ht="15">
       <c r="A16" s="4" t="s">
         <v>68</v>
       </c>
@@ -6644,7 +6644,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" ht="15">
       <c r="A17" s="4" t="s">
         <v>70</v>
       </c>
@@ -6680,7 +6680,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="27.6">
+    <row r="18" spans="1:11" ht="29.25">
       <c r="A18" s="4" t="s">
         <v>72</v>
       </c>
@@ -6716,7 +6716,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" ht="15">
       <c r="A19" s="4" t="s">
         <v>74</v>
       </c>
@@ -6752,7 +6752,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="27.6">
+    <row r="20" spans="1:11" ht="29.25">
       <c r="A20" s="4" t="s">
         <v>76</v>
       </c>
@@ -6788,7 +6788,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="27.6">
+    <row r="21" spans="1:11" ht="29.25">
       <c r="A21" s="4" t="s">
         <v>78</v>
       </c>
@@ -6824,7 +6824,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="27.6">
+    <row r="22" spans="1:11" ht="29.25">
       <c r="A22" s="4" t="s">
         <v>80</v>
       </c>
@@ -6860,7 +6860,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" ht="15">
       <c r="A23" s="4" t="s">
         <v>82</v>
       </c>
@@ -6942,9 +6942,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="25.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -6956,7 +6956,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>227</v>
       </c>
@@ -6971,7 +6971,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -6989,7 +6989,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -7007,7 +7007,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -7025,7 +7025,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -7043,7 +7043,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -7100,7 +7100,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" ht="15">
       <c r="A10" s="4" t="s">
         <v>84</v>
       </c>
@@ -7136,7 +7136,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="27.6">
+    <row r="11" spans="1:11" ht="29.25">
       <c r="A11" s="4" t="s">
         <v>86</v>
       </c>
@@ -7172,7 +7172,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" ht="15">
       <c r="A12" s="4" t="s">
         <v>88</v>
       </c>
@@ -7208,7 +7208,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" ht="15">
       <c r="A13" s="4" t="s">
         <v>90</v>
       </c>
@@ -7244,7 +7244,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" ht="15">
       <c r="A14" s="4" t="s">
         <v>92</v>
       </c>
@@ -7280,7 +7280,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" ht="15">
       <c r="A15" s="4" t="s">
         <v>94</v>
       </c>
@@ -7316,7 +7316,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" ht="29.25">
       <c r="A16" s="4" t="s">
         <v>96</v>
       </c>
@@ -7352,7 +7352,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" ht="15">
       <c r="A17" s="4" t="s">
         <v>98</v>
       </c>
@@ -7388,7 +7388,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" ht="15">
       <c r="A18" s="4" t="s">
         <v>100</v>
       </c>
@@ -7424,7 +7424,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="27.6">
+    <row r="19" spans="1:11" ht="29.25">
       <c r="A19" s="4" t="s">
         <v>102</v>
       </c>
@@ -7501,7 +7501,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -7515,7 +7515,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>232</v>
       </c>
@@ -7530,7 +7530,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -7548,7 +7548,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -7566,7 +7566,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -7584,7 +7584,7 @@
         <v>22.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -7602,7 +7602,7 @@
         <v>21.5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -7659,7 +7659,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" ht="15">
       <c r="A10" s="4" t="s">
         <v>104</v>
       </c>
@@ -7695,7 +7695,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" ht="15">
       <c r="A11" s="4" t="s">
         <v>106</v>
       </c>
@@ -7731,7 +7731,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" ht="15">
       <c r="A12" s="4" t="s">
         <v>108</v>
       </c>
@@ -7767,7 +7767,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" ht="15">
       <c r="A13" s="4" t="s">
         <v>110</v>
       </c>
@@ -7803,7 +7803,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" ht="15">
       <c r="A14" s="4" t="s">
         <v>112</v>
       </c>
@@ -7839,7 +7839,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" ht="15">
       <c r="A15" s="4" t="s">
         <v>114</v>
       </c>
@@ -7875,7 +7875,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" ht="15">
       <c r="A16" s="4" t="s">
         <v>116</v>
       </c>
@@ -7911,7 +7911,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="27.6">
+    <row r="17" spans="1:11" ht="29.25">
       <c r="A17" s="4" t="s">
         <v>118</v>
       </c>
@@ -7947,7 +7947,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="27.6">
+    <row r="18" spans="1:11" ht="29.25">
       <c r="A18" s="4" t="s">
         <v>120</v>
       </c>
@@ -7983,7 +7983,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="27.6">
+    <row r="19" spans="1:11" ht="29.25">
       <c r="A19" s="4" t="s">
         <v>122</v>
       </c>
@@ -8065,9 +8065,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="23.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -8079,7 +8079,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>236</v>
       </c>
@@ -8094,7 +8094,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -8112,7 +8112,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -8127,10 +8127,10 @@
       </c>
       <c r="H3" s="2">
         <f>COUNTIF(H10:H27,"Finalizado")</f>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="16.8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -8148,7 +8148,7 @@
         <v>24.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -8163,16 +8163,16 @@
       </c>
       <c r="H5" s="2">
         <f>SUM(F10:F27)</f>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="16.8">
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
       <c r="H6" s="2">
         <f>SUM(G10:G27)</f>
-        <v>7.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -8223,7 +8223,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="27.6">
+    <row r="10" spans="1:11" ht="29.25">
       <c r="A10" s="4" t="s">
         <v>124</v>
       </c>
@@ -8255,9 +8255,11 @@
       <c r="J10" s="5">
         <v>46309</v>
       </c>
-      <c r="K10" s="4"/>
-    </row>
-    <row r="11" spans="1:11">
+      <c r="K10" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15">
       <c r="A11" s="4" t="s">
         <v>126</v>
       </c>
@@ -8289,9 +8291,11 @@
       <c r="J11" s="5">
         <v>46309</v>
       </c>
-      <c r="K11" s="4"/>
-    </row>
-    <row r="12" spans="1:11" ht="27.6">
+      <c r="K11" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="29.25">
       <c r="A12" s="4" t="s">
         <v>128</v>
       </c>
@@ -8323,9 +8327,11 @@
       <c r="J12" s="5">
         <v>46309</v>
       </c>
-      <c r="K12" s="4"/>
-    </row>
-    <row r="13" spans="1:11">
+      <c r="K12" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15">
       <c r="A13" s="4" t="s">
         <v>130</v>
       </c>
@@ -8357,9 +8363,11 @@
       <c r="J13" s="5">
         <v>46309</v>
       </c>
-      <c r="K13" s="4"/>
-    </row>
-    <row r="14" spans="1:11" ht="27.6">
+      <c r="K13" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="29.25">
       <c r="A14" s="4" t="s">
         <v>132</v>
       </c>
@@ -8391,9 +8399,11 @@
       <c r="J14" s="5">
         <v>46309</v>
       </c>
-      <c r="K14" s="4"/>
-    </row>
-    <row r="15" spans="1:11">
+      <c r="K14" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15">
       <c r="A15" s="4" t="s">
         <v>134</v>
       </c>
@@ -8425,9 +8435,11 @@
       <c r="J15" s="5">
         <v>46309</v>
       </c>
-      <c r="K15" s="4"/>
-    </row>
-    <row r="16" spans="1:11">
+      <c r="K15" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="15">
       <c r="A16" s="4" t="s">
         <v>136</v>
       </c>
@@ -8459,9 +8471,11 @@
       <c r="J16" s="5">
         <v>46309</v>
       </c>
-      <c r="K16" s="4"/>
-    </row>
-    <row r="17" spans="1:11">
+      <c r="K16" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="15">
       <c r="A17" s="4" t="s">
         <v>138</v>
       </c>
@@ -8493,9 +8507,11 @@
       <c r="J17" s="5">
         <v>46313</v>
       </c>
-      <c r="K17" s="4"/>
-    </row>
-    <row r="18" spans="1:11">
+      <c r="K17" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="15">
       <c r="A18" s="4" t="s">
         <v>140</v>
       </c>
@@ -8527,9 +8543,11 @@
       <c r="J18" s="5">
         <v>46313</v>
       </c>
-      <c r="K18" s="4"/>
-    </row>
-    <row r="19" spans="1:11">
+      <c r="K18" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="15">
       <c r="A19" s="4" t="s">
         <v>142</v>
       </c>
@@ -8561,9 +8579,11 @@
       <c r="J19" s="5">
         <v>46313</v>
       </c>
-      <c r="K19" s="4"/>
-    </row>
-    <row r="20" spans="1:11">
+      <c r="K19" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="15">
       <c r="A20" s="4" t="s">
         <v>144</v>
       </c>
@@ -8595,9 +8615,11 @@
       <c r="J20" s="5">
         <v>46313</v>
       </c>
-      <c r="K20" s="4"/>
-    </row>
-    <row r="21" spans="1:11">
+      <c r="K20" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15">
       <c r="A21" s="4" t="s">
         <v>146</v>
       </c>
@@ -8629,9 +8651,11 @@
       <c r="J21" s="5">
         <v>46313</v>
       </c>
-      <c r="K21" s="4"/>
-    </row>
-    <row r="22" spans="1:11">
+      <c r="K21" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="15">
       <c r="A22" s="4" t="s">
         <v>148</v>
       </c>
@@ -8663,9 +8687,11 @@
       <c r="J22" s="5">
         <v>46313</v>
       </c>
-      <c r="K22" s="4"/>
-    </row>
-    <row r="23" spans="1:11">
+      <c r="K22" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15">
       <c r="A23" s="4" t="s">
         <v>150</v>
       </c>
@@ -8681,19 +8707,27 @@
       <c r="E23" s="6">
         <v>1.5</v>
       </c>
-      <c r="F23" s="6"/>
+      <c r="F23" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G23" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="4"/>
-    </row>
-    <row r="24" spans="1:11">
+        <v>220</v>
+      </c>
+      <c r="I23" s="5">
+        <v>46316</v>
+      </c>
+      <c r="J23" s="5">
+        <v>46317</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="15">
       <c r="A24" s="4" t="s">
         <v>152</v>
       </c>
@@ -8709,19 +8743,27 @@
       <c r="E24" s="6">
         <v>1.5</v>
       </c>
-      <c r="F24" s="6"/>
+      <c r="F24" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G24" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="4"/>
-    </row>
-    <row r="25" spans="1:11">
+        <v>220</v>
+      </c>
+      <c r="I24" s="5">
+        <v>46316</v>
+      </c>
+      <c r="J24" s="5">
+        <v>46317</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="15">
       <c r="A25" s="4" t="s">
         <v>154</v>
       </c>
@@ -8737,19 +8779,27 @@
       <c r="E25" s="6">
         <v>1.5</v>
       </c>
-      <c r="F25" s="6"/>
+      <c r="F25" s="6">
+        <v>1.5</v>
+      </c>
       <c r="G25" s="6">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="4"/>
-    </row>
-    <row r="26" spans="1:11" ht="27.6">
+        <v>220</v>
+      </c>
+      <c r="I25" s="5">
+        <v>46316</v>
+      </c>
+      <c r="J25" s="5">
+        <v>46317</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="29.25">
       <c r="A26" s="4" t="s">
         <v>156</v>
       </c>
@@ -8765,19 +8815,27 @@
       <c r="E26" s="6">
         <v>1</v>
       </c>
-      <c r="F26" s="6"/>
+      <c r="F26" s="6">
+        <v>1</v>
+      </c>
       <c r="G26" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="4"/>
-    </row>
-    <row r="27" spans="1:11" ht="27.6">
+        <v>220</v>
+      </c>
+      <c r="I26" s="5">
+        <v>46316</v>
+      </c>
+      <c r="J26" s="5">
+        <v>46317</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="29.25">
       <c r="A27" s="4" t="s">
         <v>158</v>
       </c>
@@ -8793,17 +8851,25 @@
       <c r="E27" s="6">
         <v>2</v>
       </c>
-      <c r="F27" s="6"/>
+      <c r="F27" s="6">
+        <v>2</v>
+      </c>
       <c r="G27" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="4"/>
+        <v>220</v>
+      </c>
+      <c r="I27" s="5">
+        <v>46316</v>
+      </c>
+      <c r="J27" s="5">
+        <v>46317</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>247</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -8814,7 +8880,7 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <conditionalFormatting sqref="F17:F27">
+  <conditionalFormatting sqref="F17:F22">
     <cfRule type="expression" dxfId="9" priority="5">
       <formula>AND($H17="Finalizado",$F17="")</formula>
     </cfRule>
@@ -8851,9 +8917,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K29"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="23.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
@@ -8865,7 +8931,7 @@
     <col min="11" max="11" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.9" customHeight="1">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>241</v>
       </c>
@@ -8880,7 +8946,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="16.8">
+    <row r="2" spans="1:11" ht="16.5">
       <c r="A2" s="7" t="s">
         <v>201</v>
       </c>
@@ -8898,7 +8964,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.8">
+    <row r="3" spans="1:11" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>203</v>
       </c>
@@ -8916,7 +8982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.8">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>205</v>
       </c>
@@ -8934,7 +9000,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="7" t="s">
         <v>248</v>
       </c>
@@ -8952,7 +9018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="G6" s="1" t="s">
         <v>210</v>
       </c>
@@ -9061,7 +9127,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" ht="28.5">
       <c r="A12" s="4" t="s">
         <v>164</v>
       </c>
@@ -9165,7 +9231,7 @@
       <c r="J15" s="5"/>
       <c r="K15" s="4"/>
     </row>
-    <row r="16" spans="1:11" ht="27.6">
+    <row r="16" spans="1:11" ht="28.5">
       <c r="A16" s="4" t="s">
         <v>172</v>
       </c>
@@ -9217,7 +9283,7 @@
       <c r="J17" s="5"/>
       <c r="K17" s="4"/>
     </row>
-    <row r="18" spans="1:11" ht="27.6">
+    <row r="18" spans="1:11" ht="28.5">
       <c r="A18" s="4" t="s">
         <v>176</v>
       </c>
@@ -9243,7 +9309,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="4"/>
     </row>
-    <row r="19" spans="1:11" ht="27.6">
+    <row r="19" spans="1:11" ht="28.5">
       <c r="A19" s="4" t="s">
         <v>178</v>
       </c>
@@ -9373,7 +9439,7 @@
       <c r="J23" s="5"/>
       <c r="K23" s="4"/>
     </row>
-    <row r="24" spans="1:11" ht="27.6">
+    <row r="24" spans="1:11" ht="28.5">
       <c r="A24" s="4" t="s">
         <v>188</v>
       </c>
@@ -9399,7 +9465,7 @@
       <c r="J24" s="5"/>
       <c r="K24" s="4"/>
     </row>
-    <row r="25" spans="1:11" ht="27.6">
+    <row r="25" spans="1:11" ht="28.5">
       <c r="A25" s="4" t="s">
         <v>190</v>
       </c>
@@ -9451,7 +9517,7 @@
       <c r="J26" s="5"/>
       <c r="K26" s="4"/>
     </row>
-    <row r="27" spans="1:11" ht="27.6">
+    <row r="27" spans="1:11" ht="28.5">
       <c r="A27" s="4" t="s">
         <v>194</v>
       </c>

</xml_diff>